<commit_message>
Managers Report we 2026-05-09
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -5929,7 +5929,9 @@
       </c>
       <c r="B13" s="156" t="n"/>
       <c r="C13" s="157" t="n"/>
-      <c r="D13" s="158" t="n"/>
+      <c r="D13" s="158" t="n">
+        <v>102500.77</v>
+      </c>
       <c r="E13" s="159" t="n">
         <v>7470.97584</v>
       </c>
@@ -6108,7 +6110,9 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n"/>
-      <c r="D16" s="167" t="n"/>
+      <c r="D16" s="167" t="n">
+        <v>10553.06</v>
+      </c>
       <c r="E16" s="168" t="n">
         <v>12623.25</v>
       </c>
@@ -6171,7 +6175,9 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n"/>
-      <c r="D17" s="168" t="n"/>
+      <c r="D17" s="168" t="n">
+        <v>1275.48</v>
+      </c>
       <c r="E17" s="168" t="n">
         <v>1583.68</v>
       </c>
@@ -6231,7 +6237,9 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n"/>
-      <c r="D18" s="167" t="n"/>
+      <c r="D18" s="167" t="n">
+        <v>1486.35</v>
+      </c>
       <c r="E18" s="168" t="n">
         <v>1519.64</v>
       </c>
@@ -6291,7 +6299,9 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n"/>
-      <c r="D19" s="167" t="n"/>
+      <c r="D19" s="167" t="n">
+        <v>843.39</v>
+      </c>
       <c r="E19" s="168" t="n">
         <v>1153.34</v>
       </c>
@@ -6351,7 +6361,9 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n"/>
-      <c r="D20" s="168" t="n"/>
+      <c r="D20" s="168" t="n">
+        <v>3004.79</v>
+      </c>
       <c r="E20" s="168" t="n">
         <v>25441.86</v>
       </c>
@@ -6414,7 +6426,9 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n"/>
-      <c r="D21" s="167" t="n"/>
+      <c r="D21" s="167" t="n">
+        <v>2314.45</v>
+      </c>
       <c r="E21" s="168" t="n">
         <v>5301.2</v>
       </c>
@@ -6477,7 +6491,9 @@
       </c>
       <c r="B22" s="171" t="n"/>
       <c r="C22" s="172" t="n"/>
-      <c r="D22" s="168" t="n"/>
+      <c r="D22" s="168" t="n">
+        <v>9107.02000000001</v>
+      </c>
       <c r="E22" s="168" t="n">
         <v>40229.73338</v>
       </c>
@@ -6540,7 +6556,9 @@
       </c>
       <c r="B23" s="171" t="n"/>
       <c r="C23" s="172" t="n"/>
-      <c r="D23" s="168" t="n"/>
+      <c r="D23" s="168" t="n">
+        <v>3715.48</v>
+      </c>
       <c r="E23" s="168" t="n">
         <v>8801.773020000001</v>
       </c>
@@ -6603,7 +6621,9 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n"/>
-      <c r="D24" s="175" t="n"/>
+      <c r="D24" s="175" t="n">
+        <v>162.68</v>
+      </c>
       <c r="E24" s="168" t="n">
         <v>26988.62</v>
       </c>
@@ -7499,7 +7519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7792,96 +7812,159 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Stocktake error: name 'extract_stocktake_closing_by_dept' is not defined</t>
+          <t>OK stocktake: Cigarettes = 102500.77 row 13</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 378997.66</t>
+          <t>OK stocktake: Produce = 9107.02 row 22</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 348702.09</t>
+          <t>OK stocktake: Fish = 2314.45 row 21</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1673</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 843.39 row 19</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.13</t>
+          <t>OK stocktake: Beef = 10553.06 row 16</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.18</t>
+          <t>OK stocktake: Lamb = 1275.48 row 17</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK scan margin std row 23: 0.42</t>
+          <t>OK stocktake: Pork = 1486.35 row 18</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK scan margin std row 24: 0.19</t>
+          <t>OK stocktake: Poultry = 3004.79 row 20</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.20</t>
+          <t>OK stocktake: Deli = 3715.48 row 23</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.25</t>
+          <t>OK stocktake: Provisions = 162.68 row 24</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.19</t>
+          <t>OK sales inc vat G4: 378997.66</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.11</t>
+          <t>OK sales ex vat G5: 348702.09</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.17</t>
+          <t>OK margin G6: 0.1673</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 13: 0.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 22: 0.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 23: 0.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 24: 0.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 16: 0.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 17: 0.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 18: 0.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 19: 0.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 20: 0.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>OK scan margin meat row 21: 0.19</t>
         </is>

</xml_diff>

<commit_message>
Managers Report we 2026-05-16
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 9.5.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 16.5.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5727,7 +5727,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>0.169658166607818</v>
+        <v>0.179217033888259</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5924,12 +5924,14 @@
         </is>
       </c>
       <c r="B13" s="156" t="n"/>
-      <c r="C13" s="157" t="n"/>
+      <c r="C13" s="157" t="n">
+        <v>102500.77</v>
+      </c>
       <c r="D13" s="158" t="n">
-        <v>102500.77</v>
+        <v>823.9</v>
       </c>
       <c r="E13" s="159" t="n">
-        <v>1165.696320487816</v>
+        <v>1284.422104204126</v>
       </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
@@ -6104,13 +6106,13 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n">
-        <v>11190.66</v>
+        <v>10553.06</v>
       </c>
       <c r="D16" s="167" t="n">
-        <v>10553.06</v>
+        <v>9782.189999999999</v>
       </c>
       <c r="E16" s="168" t="n">
-        <v>12623.25</v>
+        <v>12520.9</v>
       </c>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
@@ -6129,7 +6131,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.200804489155919</v>
+        <v>0.205083592737876</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6171,13 +6173,13 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n">
-        <v>1218.77</v>
+        <v>1275.48</v>
       </c>
       <c r="D17" s="168" t="n">
-        <v>1275.48</v>
+        <v>1305.81</v>
       </c>
       <c r="E17" s="168" t="n">
-        <v>1583.68</v>
+        <v>1591.76</v>
       </c>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
@@ -6193,7 +6195,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.24921000088739</v>
+        <v>0.244715593540754</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6235,13 +6237,13 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n">
-        <v>1304.91</v>
+        <v>1486.35</v>
       </c>
       <c r="D18" s="167" t="n">
-        <v>1486.35</v>
+        <v>1278.54</v>
       </c>
       <c r="E18" s="168" t="n">
-        <v>1519.64</v>
+        <v>1709.43</v>
       </c>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
@@ -6257,7 +6259,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.188586862195859</v>
+        <v>0.206539820447632</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6299,13 +6301,13 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n">
-        <v>852.36</v>
+        <v>843.39</v>
       </c>
       <c r="D19" s="167" t="n">
-        <v>843.39</v>
+        <v>1044.86</v>
       </c>
       <c r="E19" s="168" t="n">
-        <v>1153.34</v>
+        <v>1125.56</v>
       </c>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
@@ -6321,7 +6323,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.114740707259225</v>
+        <v>0.116175806394878</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6363,13 +6365,13 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n">
-        <v>2411.94</v>
+        <v>3004.79</v>
       </c>
       <c r="D20" s="168" t="n">
-        <v>3004.79</v>
+        <v>2733.67</v>
       </c>
       <c r="E20" s="168" t="n">
-        <v>25441.86</v>
+        <v>25390.16</v>
       </c>
       <c r="F20" s="169">
         <f>-B35</f>
@@ -6388,7 +6390,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.169512407803833</v>
+        <v>0.16405310293873</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6430,13 +6432,13 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n">
-        <v>2146.6</v>
+        <v>2314.45</v>
       </c>
       <c r="D21" s="167" t="n">
-        <v>2314.45</v>
+        <v>2280.55</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>5301.2</v>
+        <v>6083.82</v>
       </c>
       <c r="F21" s="169">
         <f>-B36</f>
@@ -6455,7 +6457,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.186095591520898</v>
+        <v>0.191766155248264</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6497,13 +6499,13 @@
       </c>
       <c r="B22" s="171" t="n"/>
       <c r="C22" s="172" t="n">
-        <v>9261.11999999999</v>
+        <v>9107.02000000001</v>
       </c>
       <c r="D22" s="168" t="n">
-        <v>9107.02000000001</v>
+        <v>9900.54000000001</v>
       </c>
       <c r="E22" s="168" t="n">
-        <v>6555.729730104664</v>
+        <v>6547.114535375959</v>
       </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
@@ -6562,13 +6564,11 @@
       </c>
       <c r="B23" s="171" t="n"/>
       <c r="C23" s="172" t="n">
-        <v>3924.75</v>
-      </c>
-      <c r="D23" s="168" t="n">
         <v>3715.48</v>
       </c>
+      <c r="D23" s="168" t="n"/>
       <c r="E23" s="168" t="n">
-        <v>1573.74654084731</v>
+        <v>1488.517014878284</v>
       </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
@@ -6627,13 +6627,13 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n">
-        <v>135.25</v>
+        <v>162.68</v>
       </c>
       <c r="D24" s="175" t="n">
-        <v>162.68</v>
+        <v>107.03</v>
       </c>
       <c r="E24" s="168" t="n">
-        <v>4594.42314964365</v>
+        <v>4358.191001925469</v>
       </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
@@ -6868,7 +6868,7 @@
         </is>
       </c>
       <c r="I30" s="189" t="n">
-        <v>155.196</v>
+        <v>434.671</v>
       </c>
       <c r="J30" s="27" t="n"/>
     </row>
@@ -6896,7 +6896,7 @@
         </is>
       </c>
       <c r="I31" s="189" t="n">
-        <v>341.611</v>
+        <v>199.712</v>
       </c>
       <c r="J31" s="27" t="n"/>
     </row>
@@ -6924,7 +6924,7 @@
         </is>
       </c>
       <c r="I32" s="189" t="n">
-        <v>25.715</v>
+        <v>87.02500000000001</v>
       </c>
       <c r="J32" s="27" t="n"/>
     </row>
@@ -6952,7 +6952,7 @@
         </is>
       </c>
       <c r="I33" s="189" t="n">
-        <v>4.7</v>
+        <v>41.13</v>
       </c>
       <c r="J33" s="27" t="n"/>
     </row>
@@ -6980,7 +6980,7 @@
         </is>
       </c>
       <c r="I34" s="189" t="n">
-        <v>13.008</v>
+        <v>54.146</v>
       </c>
       <c r="J34" s="27" t="n"/>
     </row>
@@ -7007,7 +7007,9 @@
           <t>D0029 - Beers / Wines / Spirits</t>
         </is>
       </c>
-      <c r="I35" s="189" t="n"/>
+      <c r="I35" s="189" t="n">
+        <v>42.246</v>
+      </c>
       <c r="J35" s="27" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -7060,7 +7062,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>1125.52</v>
+        <v>1393.823</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7073,7 +7075,7 @@
         </is>
       </c>
       <c r="I38" s="162" t="n">
-        <v>776.484</v>
+        <v>841.3330000000001</v>
       </c>
       <c r="J38" s="27" t="n"/>
     </row>
@@ -7086,7 +7088,7 @@
         </is>
       </c>
       <c r="I39" s="189" t="n">
-        <v>135.377</v>
+        <v>84.06999999999999</v>
       </c>
       <c r="J39" s="27" t="n"/>
     </row>
@@ -7119,7 +7121,7 @@
         </is>
       </c>
       <c r="I40" s="189" t="n">
-        <v>39.137</v>
+        <v>93.542</v>
       </c>
       <c r="J40" s="27" t="n"/>
     </row>
@@ -7140,7 +7142,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>29.536</v>
+        <v>81.86500000000001</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7165,7 +7167,7 @@
         </is>
       </c>
       <c r="I42" s="189" t="n">
-        <v>19.604</v>
+        <v>60.268</v>
       </c>
       <c r="J42" s="27" t="n"/>
     </row>
@@ -7186,7 +7188,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>80.79000000000001</v>
+        <v>202.38</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7211,7 +7213,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>836.9100000000001</v>
+        <v>862.6469999999999</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7232,7 +7234,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>351.049</v>
+        <v>379.4</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7257,7 +7259,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>674.5</v>
+        <v>735.6320000000001</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7278,7 +7280,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>1026.485</v>
+        <v>1253.179</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7312,7 +7314,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>1394.61</v>
+        <v>1136.11</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7325,7 +7327,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>85.89600000000002</v>
+        <v>128.176</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7529,70 +7531,70 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-05-09</t>
+          <t>P&amp;L Build Log - Week Ending 2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\stocktake\Stocktake_2026-05-09.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\stocktake\Stocktake_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\opr_standard\OPR_Standard_WEEK_2026-05-09.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_standard\OPR_Standard_WEEK_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\opr_standard\OPR_Standard_DAY_2026-05-09.xlsx</t>
+          <t>Downloaded OPR_STANDARD_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_standard\OPR_Standard_DAY_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\opr_standard\OPR_Standard_SAT_2026-05-09.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_standard\OPR_Standard_SAT_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\opr_meat\OPR_Meat_WEEK_2026-05-09.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_meat\OPR_Meat_WEEK_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\opr_meat\OPR_Meat_DAY_2026-05-09.xlsx</t>
+          <t>Downloaded OPR_MEAT_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_meat\OPR_Meat_DAY_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\opr_meat\OPR_Meat_SAT_2026-05-09.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_meat\OPR_Meat_SAT_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\waste\Waste_WEEK_2026-05-09.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\waste\Waste_WEEK_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-09\waste\Waste_DAY_2026-05-09.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\waste\Waste_DAY_2026-05-16.xlsx</t>
         </is>
       </c>
     </row>
@@ -7606,322 +7608,322 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-05-02-v3.xlsx</t>
+          <t>INFO: Previous week file: Managers_Report_we_2026-05-09-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-05-02-v3.xlsx</t>
+          <t>OK opening stock from Managers_Report_we_2026-05-09-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR std: Cigarettes = 1165.70 row 13</t>
+          <t>OK OPR std: Cigarettes = 1284.42 row 13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR std: Produce = 6555.73 row 22</t>
+          <t>OK OPR std: Produce = 6547.11 row 22</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR std: Deli = 1573.75 row 23</t>
+          <t>OK OPR std: Deli = 1488.52 row 23</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR std: Provisions = 4594.42 row 24</t>
+          <t>OK OPR std: Provisions = 4358.19 row 24</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OK OPR meat: Beef = 12623.25 row 16</t>
+          <t>OK OPR meat: Beef = 12520.90 row 16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OK OPR meat: Lamb = 1583.68 row 17</t>
+          <t>OK OPR meat: Lamb = 1591.76 row 17</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OK OPR meat: Pork = 1519.64 row 18</t>
+          <t>OK OPR meat: Pork = 1709.43 row 18</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OK OPR meat: Bacon &amp; Loose S.R.P = 1153.34 row 19</t>
+          <t>OK OPR meat: Bacon &amp; Loose S.R.P = 1125.56 row 19</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>OK OPR meat: Poultry = 25441.86 row 20</t>
+          <t>OK OPR meat: Poultry = 25390.16 row 20</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>OK OPR meat: Fish = 5301.20 row 21</t>
+          <t>OK OPR meat: Fish = 6083.82 row 21</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>OK waste: grocery_impulse = 155.20 row 30</t>
+          <t>OK waste: grocery_impulse = 434.67 row 30</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OK waste: grocery_edible = 341.61 row 31</t>
+          <t>OK waste: grocery_edible = 199.71 row 31</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OK waste: grocery_non_food = 25.71 row 32</t>
+          <t>OK waste: grocery_non_food = 87.03 row 32</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OK waste: baby_kids = 4.70 row 33</t>
+          <t>OK waste: baby_kids = 41.13 row 33</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 1125.52 row 37</t>
+          <t>OK waste: personal_care = 54.15 row 34</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>OK waste: meat_total = 776.48 row 38</t>
+          <t>OK waste: beer_wine_spirits = 42.25 row 35</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 836.91 row 44</t>
+          <t>OK waste: Produce = 1393.82 row 37</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 351.05 row 45</t>
+          <t>OK waste: meat_total = 841.33 row 38</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 674.50 row 46</t>
+          <t>OK waste: Fish = 862.65 row 44</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 1026.48 row 47</t>
+          <t>OK waste: Bacon = 60.27 row 42</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 1394.61 row 48</t>
+          <t>OK waste: dairy = 379.40 row 45</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 85.90 row 49</t>
+          <t>OK waste: bread_cakes = 735.63 row 46</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK waste: Beef = 135.38 row 39</t>
+          <t>OK waste: Deli = 1253.18 row 47</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK waste: Lamb = 39.14 row 40</t>
+          <t>OK waste: Provisions = 1136.11 row 48</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 29.54 row 41</t>
+          <t>OK waste: frozen = 128.18 row 49</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK waste: Bacon = 19.60 row 42</t>
+          <t>OK waste: Beef = 84.07 row 39</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 80.79 row 43</t>
+          <t>OK waste: Lamb = 93.54 row 40</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK waste: personal_care = 13.01 row 34</t>
+          <t>OK waste: Pork = 81.87 row 41</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK stocktake: Cigarettes = 102500.77 row 13</t>
+          <t>OK waste: Poultry = 202.38 row 43</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK stocktake: Produce = 9107.02 row 22</t>
+          <t>OK stocktake: Cigarettes = 823.90 row 13</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 2314.45 row 21</t>
+          <t>OK stocktake: Produce = 9900.54 row 22</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 843.39 row 19</t>
+          <t>OK stocktake: Fish = 2280.55 row 21</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 10553.06 row 16</t>
+          <t>OK stocktake: Beef = 9782.19 row 16</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 1275.48 row 17</t>
+          <t>OK stocktake: Lamb = 1305.81 row 17</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 1486.35 row 18</t>
+          <t>OK stocktake: Pork = 1278.54 row 18</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 3004.79 row 20</t>
+          <t>OK stocktake: Poultry = 2733.67 row 20</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK stocktake: Deli = 3715.48 row 23</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 1044.86 row 19</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 162.68 row 24</t>
+          <t>OK stocktake: Provisions = 107.03 row 24</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 0.17</t>
+          <t>OK sales ex vat G5: 0.18</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.20</t>
+          <t>OK scan margin meat row 16: 0.21</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.25</t>
+          <t>OK scan margin meat row 17: 0.24</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.19</t>
+          <t>OK scan margin meat row 18: 0.21</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.11</t>
+          <t>OK scan margin meat row 19: 0.12</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.17</t>
+          <t>OK scan margin meat row 20: 0.16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Manual push we 2026-05-16
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -5713,9 +5713,7 @@
       </c>
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
-      <c r="G4" s="150" t="n">
-        <v>368436.45</v>
-      </c>
+      <c r="G4" s="150" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="5" t="n"/>
@@ -5729,7 +5727,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>340018.57336</v>
+        <v>0.179217033888259</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5742,9 +5740,7 @@
       </c>
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
-      <c r="G6" s="38" t="n">
-        <v>0.175269942289014</v>
-      </c>
+      <c r="G6" s="38" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -5950,9 +5946,7 @@
         <f>+H13/E13</f>
         <v/>
       </c>
-      <c r="J13" s="39" t="n">
-        <v>0.12371212588697</v>
-      </c>
+      <c r="J13" s="39" t="n"/>
       <c r="K13" s="162">
         <f>E13*L13</f>
         <v/>
@@ -6529,9 +6523,7 @@
         <f>+H22/E22</f>
         <v/>
       </c>
-      <c r="J22" s="39" t="n">
-        <v>0.191284635873608</v>
-      </c>
+      <c r="J22" s="39" t="n"/>
       <c r="K22" s="162">
         <f>E22*L22</f>
         <v/>
@@ -6594,9 +6586,7 @@
         <f>+H23/E23</f>
         <v/>
       </c>
-      <c r="J23" s="39" t="n">
-        <v>0.415147275490546</v>
-      </c>
+      <c r="J23" s="39" t="n"/>
       <c r="K23" s="162">
         <f>E23*L23</f>
         <v/>
@@ -6661,9 +6651,7 @@
         <f>+H24/E24</f>
         <v/>
       </c>
-      <c r="J24" s="39" t="n">
-        <v>0.197147435548971</v>
-      </c>
+      <c r="J24" s="39" t="n"/>
       <c r="K24" s="162">
         <f>E24*L24</f>
         <v/>
@@ -7537,7 +7525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A65"/>
+  <dimension ref="A1:A59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7900,89 +7888,47 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 368436.45</t>
+          <t>OK sales ex vat G5: 0.18</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 340018.57</t>
+          <t>OK scan margin meat row 16: 0.21</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1753</t>
+          <t>OK scan margin meat row 17: 0.24</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.12</t>
+          <t>OK scan margin meat row 18: 0.21</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.19</t>
+          <t>OK scan margin meat row 19: 0.12</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>OK scan margin std row 23: 0.42</t>
+          <t>OK scan margin meat row 20: 0.16</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
-        <is>
-          <t>OK scan margin std row 24: 0.20</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 16: 0.21</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 17: 0.24</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 18: 0.21</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 19: 0.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 20: 0.16</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
         <is>
           <t>OK scan margin meat row 21: 0.19</t>
         </is>

</xml_diff>

<commit_message>
Managers Report we 2026-05-23
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 16.5.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 23.5.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5714,7 +5714,7 @@
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
       <c r="G4" s="150" t="n">
-        <v>368436.45</v>
+        <v>369339.93</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -5729,7 +5729,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>340018.57336</v>
+        <v>340453.63588</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5743,7 +5743,7 @@
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
       <c r="G6" s="38" t="n">
-        <v>0.175269942289014</v>
+        <v>0.177118912283417</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5929,13 +5929,11 @@
       </c>
       <c r="B13" s="156" t="n"/>
       <c r="C13" s="157" t="n">
-        <v>102500.77</v>
-      </c>
-      <c r="D13" s="158" t="n">
-        <v>823.9</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D13" s="158" t="n"/>
       <c r="E13" s="159" t="n">
-        <v>1284.422104204126</v>
+        <v>6274.43116</v>
       </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
@@ -5951,7 +5949,7 @@
         <v/>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0.12371212588697</v>
+        <v>0.12775337988456</v>
       </c>
       <c r="K13" s="162">
         <f>E13*L13</f>
@@ -6112,14 +6110,12 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n">
-        <v>10553.06</v>
+        <v>11543</v>
       </c>
       <c r="D16" s="167" t="n">
-        <v>9782.189999999999</v>
-      </c>
-      <c r="E16" s="168" t="n">
-        <v>12520.9</v>
-      </c>
+        <v>9941.460000000001</v>
+      </c>
+      <c r="E16" s="168" t="n"/>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
         <v/>
@@ -6137,7 +6133,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.205083592737876</v>
+        <v>0.198516248713556</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6179,14 +6175,12 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n">
-        <v>1275.48</v>
+        <v>1306</v>
       </c>
       <c r="D17" s="168" t="n">
-        <v>1305.81</v>
-      </c>
-      <c r="E17" s="168" t="n">
-        <v>1591.76</v>
-      </c>
+        <v>1402.26</v>
+      </c>
+      <c r="E17" s="168" t="n"/>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
         <f>B17+C17-D17+F17</f>
@@ -6201,7 +6195,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.244715593540754</v>
+        <v>0.236689413405039</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6243,14 +6237,12 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n">
-        <v>1486.35</v>
+        <v>1478</v>
       </c>
       <c r="D18" s="167" t="n">
-        <v>1278.54</v>
-      </c>
-      <c r="E18" s="168" t="n">
-        <v>1709.43</v>
-      </c>
+        <v>888.49</v>
+      </c>
+      <c r="E18" s="168" t="n"/>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
         <f>B18+C18-D18+F18</f>
@@ -6265,7 +6257,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.206539820447632</v>
+        <v>0.221973297793405</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6307,14 +6299,12 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n">
-        <v>843.39</v>
+        <v>909</v>
       </c>
       <c r="D19" s="167" t="n">
-        <v>1044.86</v>
-      </c>
-      <c r="E19" s="168" t="n">
-        <v>1125.56</v>
-      </c>
+        <v>809.3499999999999</v>
+      </c>
+      <c r="E19" s="168" t="n"/>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
         <f>B19+C19-D19+F19</f>
@@ -6329,7 +6319,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.116175806394878</v>
+        <v>0.103764585454854</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6371,14 +6361,12 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n">
-        <v>3004.79</v>
+        <v>2961</v>
       </c>
       <c r="D20" s="168" t="n">
-        <v>2733.67</v>
-      </c>
-      <c r="E20" s="168" t="n">
-        <v>25390.16</v>
-      </c>
+        <v>3094.59</v>
+      </c>
+      <c r="E20" s="168" t="n"/>
       <c r="F20" s="169">
         <f>-B35</f>
         <v/>
@@ -6396,7 +6384,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.16405310293873</v>
+        <v>0.165764767934097</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6438,14 +6426,12 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n">
-        <v>2314.45</v>
+        <v>2683</v>
       </c>
       <c r="D21" s="167" t="n">
-        <v>2280.55</v>
-      </c>
-      <c r="E21" s="168" t="n">
-        <v>6083.82</v>
-      </c>
+        <v>2515.61</v>
+      </c>
+      <c r="E21" s="168" t="n"/>
       <c r="F21" s="169">
         <f>-B36</f>
         <v/>
@@ -6463,7 +6449,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.191766155248264</v>
+        <v>0.157967671354369</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6505,13 +6491,13 @@
       </c>
       <c r="B22" s="171" t="n"/>
       <c r="C22" s="172" t="n">
-        <v>9107.02000000001</v>
+        <v>9901</v>
       </c>
       <c r="D22" s="168" t="n">
-        <v>9900.54000000001</v>
+        <v>8957.870000000001</v>
       </c>
       <c r="E22" s="168" t="n">
-        <v>6547.114535375959</v>
+        <v>33731.20373</v>
       </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
@@ -6530,7 +6516,7 @@
         <v/>
       </c>
       <c r="J22" s="39" t="n">
-        <v>0.191284635873608</v>
+        <v>0.192713958665047</v>
       </c>
       <c r="K22" s="162">
         <f>E22*L22</f>
@@ -6572,11 +6558,13 @@
       </c>
       <c r="B23" s="171" t="n"/>
       <c r="C23" s="172" t="n">
-        <v>3715.48</v>
-      </c>
-      <c r="D23" s="168" t="n"/>
+        <v>3662</v>
+      </c>
+      <c r="D23" s="168" t="n">
+        <v>3552.36</v>
+      </c>
       <c r="E23" s="168" t="n">
-        <v>1488.517014878284</v>
+        <v>7051.02226</v>
       </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
@@ -6595,7 +6583,7 @@
         <v/>
       </c>
       <c r="J23" s="39" t="n">
-        <v>0.415147275490546</v>
+        <v>0.429769519215452</v>
       </c>
       <c r="K23" s="162">
         <f>E23*L23</f>
@@ -6637,13 +6625,13 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n">
-        <v>162.68</v>
+        <v>10872</v>
       </c>
       <c r="D24" s="175" t="n">
-        <v>107.03</v>
+        <v>250.05</v>
       </c>
       <c r="E24" s="168" t="n">
-        <v>4358.191001925469</v>
+        <v>21347.48</v>
       </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
@@ -6662,7 +6650,7 @@
         <v/>
       </c>
       <c r="J24" s="39" t="n">
-        <v>0.197147435548971</v>
+        <v>0.19960311552438</v>
       </c>
       <c r="K24" s="162">
         <f>E24*L24</f>
@@ -6880,7 +6868,7 @@
         </is>
       </c>
       <c r="I30" s="189" t="n">
-        <v>434.671</v>
+        <v>652.038</v>
       </c>
       <c r="J30" s="27" t="n"/>
     </row>
@@ -6908,7 +6896,7 @@
         </is>
       </c>
       <c r="I31" s="189" t="n">
-        <v>199.712</v>
+        <v>13.344</v>
       </c>
       <c r="J31" s="27" t="n"/>
     </row>
@@ -6936,7 +6924,7 @@
         </is>
       </c>
       <c r="I32" s="189" t="n">
-        <v>87.02500000000001</v>
+        <v>148.636</v>
       </c>
       <c r="J32" s="27" t="n"/>
     </row>
@@ -6964,7 +6952,7 @@
         </is>
       </c>
       <c r="I33" s="189" t="n">
-        <v>41.13</v>
+        <v>72.86</v>
       </c>
       <c r="J33" s="27" t="n"/>
     </row>
@@ -7020,7 +7008,7 @@
         </is>
       </c>
       <c r="I35" s="189" t="n">
-        <v>42.246</v>
+        <v>31.278</v>
       </c>
       <c r="J35" s="27" t="n"/>
     </row>
@@ -7074,7 +7062,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>1393.823</v>
+        <v>1172.333</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7087,7 +7075,7 @@
         </is>
       </c>
       <c r="I38" s="162" t="n">
-        <v>841.3330000000001</v>
+        <v>756.7850000000001</v>
       </c>
       <c r="J38" s="27" t="n"/>
     </row>
@@ -7100,7 +7088,7 @@
         </is>
       </c>
       <c r="I39" s="189" t="n">
-        <v>84.06999999999999</v>
+        <v>282.115</v>
       </c>
       <c r="J39" s="27" t="n"/>
     </row>
@@ -7133,7 +7121,7 @@
         </is>
       </c>
       <c r="I40" s="189" t="n">
-        <v>93.542</v>
+        <v>108.81</v>
       </c>
       <c r="J40" s="27" t="n"/>
     </row>
@@ -7154,7 +7142,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>81.86500000000001</v>
+        <v>166.327</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7179,7 +7167,7 @@
         </is>
       </c>
       <c r="I42" s="189" t="n">
-        <v>60.268</v>
+        <v>127.658</v>
       </c>
       <c r="J42" s="27" t="n"/>
     </row>
@@ -7200,7 +7188,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>202.38</v>
+        <v>190.2</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7225,7 +7213,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>862.6469999999999</v>
+        <v>874.046</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7246,7 +7234,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>379.4</v>
+        <v>372.621</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7271,7 +7259,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>735.6320000000001</v>
+        <v>916.991</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7292,7 +7280,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>1253.179</v>
+        <v>1250.608</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7326,7 +7314,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>1136.11</v>
+        <v>1223.48</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7339,7 +7327,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>128.176</v>
+        <v>146.224</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7537,454 +7525,398 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A65"/>
+  <dimension ref="A1:A57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-05-16</t>
+          <t>P&amp;L Build Log - Week Ending 2026-05-23</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\stocktake\Stocktake_2026-05-16.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\stocktake\Stocktake_2026-05-23.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_standard\OPR_Standard_WEEK_2026-05-16.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_standard\OPR_Standard_WEEK_2026-05-23.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_standard\OPR_Standard_DAY_2026-05-16.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_standard\OPR_Standard_SAT_2026-05-23.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_standard\OPR_Standard_SAT_2026-05-16.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_meat\OPR_Meat_WEEK_2026-05-23.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_meat\OPR_Meat_WEEK_2026-05-16.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_meat\OPR_Meat_SAT_2026-05-23.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_meat\OPR_Meat_DAY_2026-05-16.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\waste\Waste_WEEK_2026-05-23.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\opr_meat\OPR_Meat_SAT_2026-05-16.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\waste\Waste_WEEK_2026-05-16.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\waste\Waste_DAY_2026-05-23.xlsx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-16\waste\Waste_DAY_2026-05-16.xlsx</t>
+          <t>INFO: No Supabase key - purchases skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>INFO: Previous week file: Managers_Report_we_2026-05-16-v2.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INFO: No Supabase key - purchases skipped</t>
+          <t>OK opening stock from Managers_Report_we_2026-05-16-v2.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-05-09-v3.xlsx</t>
+          <t>OK OPR std: Cigarettes = 6274.43 row 13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-05-09-v3.xlsx</t>
+          <t>OK OPR std: Produce = 33731.20 row 22</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR std: Cigarettes = 1284.42 row 13</t>
+          <t>OK OPR std: Deli = 7051.02 row 23</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR std: Produce = 6547.11 row 22</t>
+          <t>OK OPR std: Provisions = 21347.48 row 24</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR std: Deli = 1488.52 row 23</t>
+          <t>OK waste: grocery_impulse = 652.04 row 30</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR std: Provisions = 4358.19 row 24</t>
+          <t>OK waste: grocery_edible = 13.34 row 31</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OK OPR meat: Beef = 12520.90 row 16</t>
+          <t>OK waste: grocery_non_food = 148.64 row 32</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OK OPR meat: Lamb = 1591.76 row 17</t>
+          <t>OK waste: baby_kids = 72.86 row 33</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OK OPR meat: Pork = 1709.43 row 18</t>
+          <t>OK waste: personal_care = 54.15 row 34</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OK OPR meat: Bacon &amp; Loose S.R.P = 1125.56 row 19</t>
+          <t>OK waste: beer_wine_spirits = 31.28 row 35</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>OK OPR meat: Poultry = 25390.16 row 20</t>
+          <t>OK waste: Produce = 1172.33 row 37</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>OK OPR meat: Fish = 6083.82 row 21</t>
+          <t>OK waste: meat_total = 756.79 row 38</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>OK waste: grocery_impulse = 434.67 row 30</t>
+          <t>OK waste: Fish = 874.05 row 44</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OK waste: grocery_edible = 199.71 row 31</t>
+          <t>OK waste: Bacon = 127.66 row 42</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OK waste: grocery_non_food = 87.03 row 32</t>
+          <t>OK waste: dairy = 372.62 row 45</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OK waste: baby_kids = 41.13 row 33</t>
+          <t>OK waste: bread_cakes = 916.99 row 46</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OK waste: personal_care = 54.15 row 34</t>
+          <t>OK waste: Deli = 1250.61 row 47</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>OK waste: beer_wine_spirits = 42.25 row 35</t>
+          <t>OK waste: Provisions = 1223.48 row 48</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 1393.82 row 37</t>
+          <t>OK waste: frozen = 146.22 row 49</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OK waste: meat_total = 841.33 row 38</t>
+          <t>OK waste: Beef = 282.12 row 39</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 862.65 row 44</t>
+          <t>OK waste: Lamb = 108.81 row 40</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: Bacon = 60.27 row 42</t>
+          <t>OK waste: Pork = 166.33 row 41</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 379.40 row 45</t>
+          <t>OK waste: Poultry = 190.20 row 43</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 735.63 row 46</t>
+          <t>OK stocktake: Produce = 8957.87 row 22</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 1253.18 row 47</t>
+          <t>OK stocktake: Fish = 2515.61 row 21</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 1136.11 row 48</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 809.35 row 19</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 128.18 row 49</t>
+          <t>OK stocktake: Beef = 9941.46 row 16</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK waste: Beef = 84.07 row 39</t>
+          <t>OK stocktake: Poultry = 3094.59 row 20</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OK waste: Lamb = 93.54 row 40</t>
+          <t>OK stocktake: Pork = 888.49 row 18</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 81.87 row 41</t>
+          <t>OK stocktake: Lamb = 1402.26 row 17</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 202.38 row 43</t>
+          <t>OK stocktake: Deli = 3552.36 row 23</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK stocktake: Cigarettes = 823.90 row 13</t>
+          <t>OK stocktake: Provisions = 250.05 row 24</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK stocktake: Produce = 9900.54 row 22</t>
+          <t>OK sales inc vat G4: 369339.93</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 2280.55 row 21</t>
+          <t>OK sales ex vat G5: 340453.64</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 9782.19 row 16</t>
+          <t>OK margin G6: 0.1771</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 1305.81 row 17</t>
+          <t>OK scan margin std row 13: 0.13</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 1278.54 row 18</t>
+          <t>OK scan margin std row 22: 0.19</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 2733.67 row 20</t>
+          <t>OK scan margin std row 23: 0.43</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 1044.86 row 19</t>
+          <t>OK scan margin std row 24: 0.20</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 107.03 row 24</t>
+          <t>OK scan margin meat row 16: 0.20</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 368436.45</t>
+          <t>OK scan margin meat row 17: 0.24</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 340018.57</t>
+          <t>OK scan margin meat row 18: 0.22</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1753</t>
+          <t>OK scan margin meat row 19: 0.10</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.12</t>
+          <t>OK scan margin meat row 20: 0.17</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.19</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>OK scan margin std row 23: 0.42</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>OK scan margin std row 24: 0.20</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 16: 0.21</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 17: 0.24</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 18: 0.21</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 19: 0.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 20: 0.16</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 21: 0.19</t>
+          <t>OK scan margin meat row 21: 0.16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Managers Report we 2026-05-30
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 23.5.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 30.5.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5714,7 +5714,7 @@
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
       <c r="G4" s="150" t="n">
-        <v>369339.93</v>
+        <v>401866.93</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -5729,7 +5729,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>340453.63588</v>
+        <v>368721.29426</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5743,7 +5743,7 @@
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
       <c r="G6" s="38" t="n">
-        <v>0.177118912283417</v>
+        <v>0.170042603115265</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5925,12 +5925,10 @@
         </is>
       </c>
       <c r="B13" s="156" t="n"/>
-      <c r="C13" s="157" t="n">
-        <v>0</v>
-      </c>
+      <c r="C13" s="157" t="n"/>
       <c r="D13" s="158" t="n"/>
       <c r="E13" s="159" t="n">
-        <v>7821.26047</v>
+        <v>7420.96764</v>
       </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
@@ -5946,7 +5944,7 @@
         <v/>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0.12775337988456</v>
+        <v>0.119992628077273</v>
       </c>
       <c r="K13" s="162">
         <f>E13*L13</f>
@@ -6107,13 +6105,13 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n">
-        <v>11543</v>
+        <v>9941.460000000001</v>
       </c>
       <c r="D16" s="167" t="n">
-        <v>9941.460000000001</v>
+        <v>12855.55</v>
       </c>
       <c r="E16" s="168" t="n">
-        <v>12398.52</v>
+        <v>14471.49</v>
       </c>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
@@ -6132,7 +6130,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.198516248713556</v>
+        <v>0.193901866359304</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6174,13 +6172,13 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n">
-        <v>1306</v>
+        <v>1402.26</v>
       </c>
       <c r="D17" s="168" t="n">
-        <v>1402.26</v>
+        <v>1723.52</v>
       </c>
       <c r="E17" s="168" t="n">
-        <v>1506.15</v>
+        <v>1217.01</v>
       </c>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
@@ -6196,7 +6194,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.236689413405039</v>
+        <v>0.245475115241452</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6238,13 +6236,13 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n">
-        <v>1478</v>
+        <v>888.49</v>
       </c>
       <c r="D18" s="167" t="n">
-        <v>888.49</v>
+        <v>1042.65</v>
       </c>
       <c r="E18" s="168" t="n">
-        <v>2115.93</v>
+        <v>2269.39</v>
       </c>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
@@ -6260,7 +6258,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.221973297793405</v>
+        <v>0.217060611001194</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6302,13 +6300,13 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n">
-        <v>909</v>
+        <v>809.3499999999999</v>
       </c>
       <c r="D19" s="167" t="n">
-        <v>809.3499999999999</v>
+        <v>723.87</v>
       </c>
       <c r="E19" s="168" t="n">
-        <v>989.73</v>
+        <v>930.6999999999999</v>
       </c>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
@@ -6324,7 +6322,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.103764585454854</v>
+        <v>0.105747816754222</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6366,13 +6364,13 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n">
-        <v>2961</v>
+        <v>3094.59</v>
       </c>
       <c r="D20" s="168" t="n">
-        <v>3094.59</v>
+        <v>4167.73</v>
       </c>
       <c r="E20" s="168" t="n">
-        <v>13119.98</v>
+        <v>13445.89</v>
       </c>
       <c r="F20" s="169">
         <f>-B35</f>
@@ -6391,7 +6389,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.165764767934097</v>
+        <v>0.163371851919062</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6433,13 +6431,13 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n">
-        <v>2683</v>
+        <v>2515.61</v>
       </c>
       <c r="D21" s="167" t="n">
-        <v>2515.61</v>
+        <v>2560.89</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>5818.06</v>
+        <v>6295.21</v>
       </c>
       <c r="F21" s="169">
         <f>-B36</f>
@@ -6458,7 +6456,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.157967671354369</v>
+        <v>0.13652840016457</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6500,13 +6498,11 @@
       </c>
       <c r="B22" s="171" t="n"/>
       <c r="C22" s="172" t="n">
-        <v>9901</v>
-      </c>
-      <c r="D22" s="168" t="n">
         <v>8957.870000000001</v>
       </c>
+      <c r="D22" s="168" t="n"/>
       <c r="E22" s="168" t="n">
-        <v>41226.67992</v>
+        <v>44980.95262</v>
       </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
@@ -6525,7 +6521,7 @@
         <v/>
       </c>
       <c r="J22" s="39" t="n">
-        <v>0.192713958665047</v>
+        <v>0.191000528658879</v>
       </c>
       <c r="K22" s="162">
         <f>E22*L22</f>
@@ -6567,13 +6563,13 @@
       </c>
       <c r="B23" s="171" t="n"/>
       <c r="C23" s="172" t="n">
-        <v>3662</v>
+        <v>3552.36</v>
       </c>
       <c r="D23" s="168" t="n">
-        <v>3552.36</v>
+        <v>3492.43</v>
       </c>
       <c r="E23" s="168" t="n">
-        <v>8786.338540000001</v>
+        <v>10215.18407</v>
       </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
@@ -6592,7 +6588,7 @@
         <v/>
       </c>
       <c r="J23" s="39" t="n">
-        <v>0.429769519215452</v>
+        <v>0.420256882360809</v>
       </c>
       <c r="K23" s="162">
         <f>E23*L23</f>
@@ -6634,13 +6630,13 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n">
-        <v>10872</v>
+        <v>250.05</v>
       </c>
       <c r="D24" s="175" t="n">
-        <v>250.05</v>
+        <v>247.87</v>
       </c>
       <c r="E24" s="168" t="n">
-        <v>25994.34</v>
+        <v>27146.15</v>
       </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
@@ -6659,7 +6655,7 @@
         <v/>
       </c>
       <c r="J24" s="39" t="n">
-        <v>0.19960311552438</v>
+        <v>0.197640103292732</v>
       </c>
       <c r="K24" s="162">
         <f>E24*L24</f>
@@ -7059,7 +7055,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>1172.333</v>
+        <v>1078.764</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7086,7 +7082,7 @@
         </is>
       </c>
       <c r="I39" s="189" t="n">
-        <v>282.115</v>
+        <v>418.482</v>
       </c>
       <c r="J39" s="27" t="n"/>
     </row>
@@ -7140,7 +7136,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>166.327</v>
+        <v>227.996</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7186,7 +7182,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>190.2</v>
+        <v>422.34</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7211,7 +7207,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>874.046</v>
+        <v>1009.138</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7232,7 +7228,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>372.621</v>
+        <v>319.317</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7257,7 +7253,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>916.991</v>
+        <v>910.058</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7278,7 +7274,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>1250.608</v>
+        <v>968.6850000000001</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7312,7 +7308,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>1223.48</v>
+        <v>1121.65</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7325,7 +7321,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>146.224</v>
+        <v>142.884</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7523,62 +7519,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A63"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-05-23</t>
+          <t>P&amp;L Build Log - Week Ending 2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\stocktake\Stocktake_2026-05-23.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\stocktake\Stocktake_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_standard\OPR_Standard_WEEK_2026-05-23.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_standard\OPR_Standard_WEEK_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_standard\OPR_Standard_SAT_2026-05-23.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_standard\OPR_Standard_SAT_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_meat\OPR_Meat_WEEK_2026-05-23.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_meat\OPR_Meat_WEEK_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\opr_meat\OPR_Meat_SAT_2026-05-23.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_meat\OPR_Meat_SAT_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\waste\Waste_WEEK_2026-05-23.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\waste\Waste_WEEK_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-23\waste\Waste_DAY_2026-05-23.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\waste\Waste_DAY_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
@@ -7592,84 +7588,84 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-05-16-v2.xlsx</t>
+          <t>INFO: Previous week file: Managers_Report_we_2026-05-23-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-05-16-v2.xlsx</t>
+          <t>OK opening stock from Managers_Report_we_2026-05-23-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Cigarettes = 7821.26 row 13</t>
+          <t>OK OPR std SAT: Cigarettes = 7420.97 row 13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Produce = 41226.68 row 22</t>
+          <t>OK OPR std SAT: Produce = 44980.95 row 22</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Deli = 8786.34 row 23</t>
+          <t>OK OPR std SAT: Deli = 10215.18 row 23</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Provisions = 25994.34 row 24</t>
+          <t>OK OPR std SAT: Provisions = 27146.15 row 24</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Beef = 12398.52 row 16</t>
+          <t>OK OPR meat SAT: Beef = 14471.49 row 16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Lamb = 1506.15 row 17</t>
+          <t>OK OPR meat SAT: Lamb = 1217.01 row 17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Pork = 2115.93 row 18</t>
+          <t>OK OPR meat SAT: Pork = 2269.39 row 18</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 989.73 row 19</t>
+          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 930.70 row 19</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Poultry = 13119.98 row 20</t>
+          <t>OK OPR meat SAT: Poultry = 13445.89 row 20</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Fish = 5818.06 row 21</t>
+          <t>OK OPR meat SAT: Fish = 6295.21 row 21</t>
         </is>
       </c>
     </row>
@@ -7718,7 +7714,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 1172.33 row 37</t>
+          <t>OK waste: Produce = 1078.76 row 37</t>
         </is>
       </c>
     </row>
@@ -7732,7 +7728,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 874.05 row 44</t>
+          <t>OK waste: Fish = 1009.14 row 44</t>
         </is>
       </c>
     </row>
@@ -7746,42 +7742,42 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 372.62 row 45</t>
+          <t>OK waste: dairy = 319.32 row 45</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 916.99 row 46</t>
+          <t>OK waste: bread_cakes = 910.06 row 46</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 1250.61 row 47</t>
+          <t>OK waste: Deli = 968.69 row 47</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 1223.48 row 48</t>
+          <t>OK waste: Provisions = 1121.65 row 48</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 146.22 row 49</t>
+          <t>OK waste: frozen = 142.88 row 49</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK waste: Beef = 282.12 row 39</t>
+          <t>OK waste: Beef = 418.48 row 39</t>
         </is>
       </c>
     </row>
@@ -7795,168 +7791,161 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 166.33 row 41</t>
+          <t>OK waste: Pork = 228.00 row 41</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 190.20 row 43</t>
+          <t>OK waste: Poultry = 422.34 row 43</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK stocktake: Produce = 8957.87 row 22</t>
+          <t>OK stocktake: Fish = 2560.89 row 21</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 2515.61 row 21</t>
+          <t>OK stocktake: Pork = 1042.65 row 18</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 809.35 row 19</t>
+          <t>OK stocktake: Poultry = 4167.73 row 20</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 9941.46 row 16</t>
+          <t>OK stocktake: Beef = 12855.55 row 16</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 3094.59 row 20</t>
+          <t>OK stocktake: Lamb = 1723.52 row 17</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 888.49 row 18</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 723.87 row 19</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 1402.26 row 17</t>
+          <t>OK stocktake: Deli = 3492.43 row 23</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK stocktake: Deli = 3552.36 row 23</t>
+          <t>OK stocktake: Provisions = 247.87 row 24</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 250.05 row 24</t>
+          <t>OK sales inc vat G4: 401866.93</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 369339.93</t>
+          <t>OK sales ex vat G5: 368721.29</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 340453.64</t>
+          <t>OK margin G6: 0.1700</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1771</t>
+          <t>OK scan margin std row 13: 0.12</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.13</t>
+          <t>OK scan margin std row 22: 0.19</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.19</t>
+          <t>OK scan margin std row 23: 0.42</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin std row 23: 0.43</t>
+          <t>OK scan margin std row 24: 0.20</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OK scan margin std row 24: 0.20</t>
+          <t>OK scan margin meat row 16: 0.19</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.20</t>
+          <t>OK scan margin meat row 17: 0.25</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.24</t>
+          <t>OK scan margin meat row 18: 0.22</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.22</t>
+          <t>OK scan margin meat row 19: 0.11</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.10</t>
+          <t>OK scan margin meat row 20: 0.16</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.17</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 21: 0.16</t>
+          <t>OK scan margin meat row 21: 0.14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Managers Report we 2026-06-06
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 30.5.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 6.6.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5714,7 +5714,7 @@
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
       <c r="G4" s="150" t="n">
-        <v>401866.93</v>
+        <v>370022.76</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -5729,7 +5729,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>368721.29426</v>
+        <v>340421.20168</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5743,7 +5743,7 @@
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
       <c r="G6" s="38" t="n">
-        <v>0.170042603115265</v>
+        <v>0.173946351454522</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5926,9 +5926,11 @@
       </c>
       <c r="B13" s="156" t="n"/>
       <c r="C13" s="157" t="n"/>
-      <c r="D13" s="158" t="n"/>
+      <c r="D13" s="158" t="n">
+        <v>123650.7399999999</v>
+      </c>
       <c r="E13" s="159" t="n">
-        <v>7420.96764</v>
+        <v>8075.52869</v>
       </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
@@ -5944,7 +5946,7 @@
         <v/>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0.119992628077273</v>
+        <v>0.128239036693955</v>
       </c>
       <c r="K13" s="162">
         <f>E13*L13</f>
@@ -6105,13 +6107,13 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n">
-        <v>9941.460000000001</v>
+        <v>12855.55</v>
       </c>
       <c r="D16" s="167" t="n">
-        <v>12855.55</v>
+        <v>10799.53</v>
       </c>
       <c r="E16" s="168" t="n">
-        <v>14471.49</v>
+        <v>12633.46</v>
       </c>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
@@ -6130,7 +6132,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.193901866359304</v>
+        <v>0.189964614602809</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6172,13 +6174,13 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n">
-        <v>1402.26</v>
+        <v>1723.52</v>
       </c>
       <c r="D17" s="168" t="n">
-        <v>1723.52</v>
+        <v>1065.31</v>
       </c>
       <c r="E17" s="168" t="n">
-        <v>1217.01</v>
+        <v>1249.36</v>
       </c>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
@@ -6194,7 +6196,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.245475115241452</v>
+        <v>0.25556342447333</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6236,13 +6238,13 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n">
-        <v>888.49</v>
+        <v>1042.65</v>
       </c>
       <c r="D18" s="167" t="n">
-        <v>1042.65</v>
+        <v>527.65</v>
       </c>
       <c r="E18" s="168" t="n">
-        <v>2269.39</v>
+        <v>1363.07</v>
       </c>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
@@ -6258,7 +6260,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.217060611001194</v>
+        <v>0.226605427454203</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6300,13 +6302,13 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n">
-        <v>809.3499999999999</v>
+        <v>723.87</v>
       </c>
       <c r="D19" s="167" t="n">
-        <v>723.87</v>
+        <v>595.9400000000001</v>
       </c>
       <c r="E19" s="168" t="n">
-        <v>930.6999999999999</v>
+        <v>1010.73</v>
       </c>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
@@ -6322,7 +6324,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.105747816754222</v>
+        <v>0.119135352376981</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6364,13 +6366,13 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n">
-        <v>3094.59</v>
+        <v>4167.73</v>
       </c>
       <c r="D20" s="168" t="n">
-        <v>4167.73</v>
+        <v>1953.62</v>
       </c>
       <c r="E20" s="168" t="n">
-        <v>13445.89</v>
+        <v>12936.92</v>
       </c>
       <c r="F20" s="169">
         <f>-B35</f>
@@ -6389,7 +6391,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.163371851919062</v>
+        <v>0.156396693339682</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6431,13 +6433,13 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n">
-        <v>2515.61</v>
+        <v>2560.89</v>
       </c>
       <c r="D21" s="167" t="n">
-        <v>2560.89</v>
+        <v>2243.06</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>6295.21</v>
+        <v>5599.55</v>
       </c>
       <c r="F21" s="169">
         <f>-B36</f>
@@ -6456,7 +6458,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.13652840016457</v>
+        <v>0.145110139207615</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6497,12 +6499,12 @@
         </is>
       </c>
       <c r="B22" s="171" t="n"/>
-      <c r="C22" s="172" t="n">
-        <v>8957.870000000001</v>
-      </c>
-      <c r="D22" s="168" t="n"/>
+      <c r="C22" s="172" t="n"/>
+      <c r="D22" s="168" t="n">
+        <v>9759.909999999991</v>
+      </c>
       <c r="E22" s="168" t="n">
-        <v>44980.95262</v>
+        <v>40960.14412</v>
       </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
@@ -6521,7 +6523,7 @@
         <v/>
       </c>
       <c r="J22" s="39" t="n">
-        <v>0.191000528658879</v>
+        <v>0.194713073924604</v>
       </c>
       <c r="K22" s="162">
         <f>E22*L22</f>
@@ -6563,13 +6565,13 @@
       </c>
       <c r="B23" s="171" t="n"/>
       <c r="C23" s="172" t="n">
-        <v>3552.36</v>
+        <v>3492.43</v>
       </c>
       <c r="D23" s="168" t="n">
-        <v>3492.43</v>
+        <v>4075.56</v>
       </c>
       <c r="E23" s="168" t="n">
-        <v>10215.18407</v>
+        <v>8464.122380000001</v>
       </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
@@ -6588,7 +6590,7 @@
         <v/>
       </c>
       <c r="J23" s="39" t="n">
-        <v>0.420256882360809</v>
+        <v>0.421223433444732</v>
       </c>
       <c r="K23" s="162">
         <f>E23*L23</f>
@@ -6630,13 +6632,13 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n">
-        <v>250.05</v>
+        <v>247.87</v>
       </c>
       <c r="D24" s="175" t="n">
-        <v>247.87</v>
+        <v>49.67</v>
       </c>
       <c r="E24" s="168" t="n">
-        <v>27146.15</v>
+        <v>24532.33</v>
       </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
@@ -6655,7 +6657,7 @@
         <v/>
       </c>
       <c r="J24" s="39" t="n">
-        <v>0.197640103292732</v>
+        <v>0.191982114214182</v>
       </c>
       <c r="K24" s="162">
         <f>E24*L24</f>
@@ -7055,7 +7057,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>1078.764</v>
+        <v>1763.827</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7082,7 +7084,7 @@
         </is>
       </c>
       <c r="I39" s="189" t="n">
-        <v>418.482</v>
+        <v>293.311</v>
       </c>
       <c r="J39" s="27" t="n"/>
     </row>
@@ -7115,7 +7117,7 @@
         </is>
       </c>
       <c r="I40" s="189" t="n">
-        <v>108.81</v>
+        <v>100.357</v>
       </c>
       <c r="J40" s="27" t="n"/>
     </row>
@@ -7136,7 +7138,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>227.996</v>
+        <v>154.169</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7161,7 +7163,7 @@
         </is>
       </c>
       <c r="I42" s="189" t="n">
-        <v>127.658</v>
+        <v>109.018</v>
       </c>
       <c r="J42" s="27" t="n"/>
     </row>
@@ -7182,7 +7184,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>422.34</v>
+        <v>648.74</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7207,7 +7209,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>1009.138</v>
+        <v>1625.363</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7228,7 +7230,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>319.317</v>
+        <v>284.522</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7253,7 +7255,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>910.058</v>
+        <v>764.784</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7274,7 +7276,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>968.6850000000001</v>
+        <v>1204.225</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7308,7 +7310,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>1121.65</v>
+        <v>1016.8</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7321,7 +7323,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>142.884</v>
+        <v>225.926</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7519,62 +7521,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-05-30</t>
+          <t>P&amp;L Build Log - Week Ending 2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\stocktake\Stocktake_2026-05-30.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\stocktake\Stocktake_2026-06-06.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_standard\OPR_Standard_WEEK_2026-05-30.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_standard\OPR_Standard_WEEK_2026-06-06.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_standard\OPR_Standard_SAT_2026-05-30.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_standard\OPR_Standard_SAT_2026-06-06.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_meat\OPR_Meat_WEEK_2026-05-30.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_meat\OPR_Meat_WEEK_2026-06-06.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\opr_meat\OPR_Meat_SAT_2026-05-30.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_meat\OPR_Meat_SAT_2026-06-06.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\waste\Waste_WEEK_2026-05-30.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\waste\Waste_WEEK_2026-06-06.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-05-30\waste\Waste_DAY_2026-05-30.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\waste\Waste_DAY_2026-06-06.xlsx</t>
         </is>
       </c>
     </row>
@@ -7588,84 +7590,84 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-05-23-v3.xlsx</t>
+          <t>INFO: Previous week file: Managers_Report_we_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-05-23-v3.xlsx</t>
+          <t>OK opening stock from Managers_Report_we_2026-05-30.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Cigarettes = 7420.97 row 13</t>
+          <t>OK OPR std SAT: Cigarettes = 8075.53 row 13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Produce = 44980.95 row 22</t>
+          <t>OK OPR std SAT: Produce = 40960.14 row 22</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Deli = 10215.18 row 23</t>
+          <t>OK OPR std SAT: Deli = 8464.12 row 23</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Provisions = 27146.15 row 24</t>
+          <t>OK OPR std SAT: Provisions = 24532.33 row 24</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Beef = 14471.49 row 16</t>
+          <t>OK OPR meat SAT: Beef = 12633.46 row 16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Lamb = 1217.01 row 17</t>
+          <t>OK OPR meat SAT: Lamb = 1249.36 row 17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Pork = 2269.39 row 18</t>
+          <t>OK OPR meat SAT: Pork = 1363.07 row 18</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 930.70 row 19</t>
+          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 1010.73 row 19</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Poultry = 13445.89 row 20</t>
+          <t>OK OPR meat SAT: Poultry = 12936.92 row 20</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Fish = 6295.21 row 21</t>
+          <t>OK OPR meat SAT: Fish = 5599.55 row 21</t>
         </is>
       </c>
     </row>
@@ -7700,252 +7702,266 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: personal_care row 34</t>
+          <t>SKIP waste top-section: beer_wine_spirits row 35</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: beer_wine_spirits row 35</t>
+          <t>OK waste: Produce = 1763.83 row 37</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 1078.76 row 37</t>
+          <t>SKIP waste top-section: meat_total row 38</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: meat_total row 38</t>
+          <t>OK waste: Fish = 1625.36 row 44</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 1009.14 row 44</t>
+          <t>OK waste: Bacon = 109.02 row 42</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OK waste: Bacon = 127.66 row 42</t>
+          <t>OK waste: dairy = 284.52 row 45</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 319.32 row 45</t>
+          <t>OK waste: bread_cakes = 764.78 row 46</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 910.06 row 46</t>
+          <t>OK waste: Deli = 1204.23 row 47</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 968.69 row 47</t>
+          <t>OK waste: Provisions = 1016.80 row 48</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 1121.65 row 48</t>
+          <t>OK waste: frozen = 225.93 row 49</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 142.88 row 49</t>
+          <t>OK waste: Beef = 293.31 row 39</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK waste: Beef = 418.48 row 39</t>
+          <t>OK waste: Lamb = 100.36 row 40</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OK waste: Lamb = 108.81 row 40</t>
+          <t>OK waste: Pork = 154.17 row 41</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 228.00 row 41</t>
+          <t>OK waste: Poultry = 648.74 row 43</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 422.34 row 43</t>
+          <t>SKIP waste top-section: personal_care row 34</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 2560.89 row 21</t>
+          <t>OK stocktake: Cigarettes = 123650.74 row 13</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 1042.65 row 18</t>
+          <t>OK stocktake: Produce = 9759.91 row 22</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 4167.73 row 20</t>
+          <t>OK stocktake: Fish = 2243.06 row 21</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 12855.55 row 16</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 595.94 row 19</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 1723.52 row 17</t>
+          <t>OK stocktake: Beef = 10799.53 row 16</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 723.87 row 19</t>
+          <t>OK stocktake: Lamb = 1065.31 row 17</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK stocktake: Deli = 3492.43 row 23</t>
+          <t>OK stocktake: Pork = 527.65 row 18</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 247.87 row 24</t>
+          <t>OK stocktake: Poultry = 1953.62 row 20</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 401866.93</t>
+          <t>OK stocktake: Deli = 4075.56 row 23</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 368721.29</t>
+          <t>OK stocktake: Provisions = 49.67 row 24</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1700</t>
+          <t>OK sales inc vat G4: 370022.76</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.12</t>
+          <t>OK sales ex vat G5: 340421.20</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.19</t>
+          <t>OK margin G6: 0.1739</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK scan margin std row 23: 0.42</t>
+          <t>OK scan margin std row 13: 0.13</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin std row 24: 0.20</t>
+          <t>OK scan margin std row 22: 0.19</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.19</t>
+          <t>OK scan margin std row 23: 0.42</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.25</t>
+          <t>OK scan margin std row 24: 0.19</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.22</t>
+          <t>OK scan margin meat row 16: 0.19</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.11</t>
+          <t>OK scan margin meat row 17: 0.26</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.16</t>
+          <t>OK scan margin meat row 18: 0.23</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 21: 0.14</t>
+          <t>OK scan margin meat row 19: 0.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 20: 0.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 21: 0.15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Managers Report we 2026-06-13
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 6.6.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 13.6.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5713,7 +5713,9 @@
       </c>
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
-      <c r="G4" s="150" t="n"/>
+      <c r="G4" s="150" t="n">
+        <v>367581.78</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="5" t="n"/>
@@ -5726,7 +5728,9 @@
       </c>
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
-      <c r="G5" s="150" t="n"/>
+      <c r="G5" s="150" t="n">
+        <v>338366.7843</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="n"/>
@@ -5738,7 +5742,9 @@
       </c>
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
-      <c r="G6" s="38" t="n"/>
+      <c r="G6" s="38" t="n">
+        <v>0.174070526992918</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -5920,8 +5926,12 @@
       </c>
       <c r="B13" s="156" t="n"/>
       <c r="C13" s="157" t="n"/>
-      <c r="D13" s="158" t="n"/>
-      <c r="E13" s="159" t="n"/>
+      <c r="D13" s="158" t="n">
+        <v>114751.02</v>
+      </c>
+      <c r="E13" s="159" t="n">
+        <v>7137.91078</v>
+      </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
         <f>B13+C13-D13+F13</f>
@@ -5935,7 +5945,9 @@
         <f>+H13/E13</f>
         <v/>
       </c>
-      <c r="J13" s="39" t="n"/>
+      <c r="J13" s="39" t="n">
+        <v>0.128699141571506</v>
+      </c>
       <c r="K13" s="162">
         <f>E13*L13</f>
         <v/>
@@ -6094,14 +6106,12 @@
         </is>
       </c>
       <c r="B16" s="165" t="n"/>
-      <c r="C16" s="166" t="n">
-        <v>12855.55</v>
-      </c>
+      <c r="C16" s="166" t="n"/>
       <c r="D16" s="167" t="n">
-        <v>6600.049999999999</v>
+        <v>1369.36</v>
       </c>
       <c r="E16" s="168" t="n">
-        <v>9958.34</v>
+        <v>13218.63</v>
       </c>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
@@ -6120,7 +6130,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.167671656119393</v>
+        <v>0.195678226109665</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6161,14 +6171,12 @@
         </is>
       </c>
       <c r="B17" s="171" t="n"/>
-      <c r="C17" s="172" t="n">
-        <v>1723.52</v>
-      </c>
+      <c r="C17" s="172" t="n"/>
       <c r="D17" s="168" t="n">
-        <v>635.54</v>
+        <v>260.86</v>
       </c>
       <c r="E17" s="168" t="n">
-        <v>964.73</v>
+        <v>1562.31</v>
       </c>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
@@ -6184,7 +6192,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.260893047795756</v>
+        <v>0.247975696244663</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6225,14 +6233,12 @@
         </is>
       </c>
       <c r="B18" s="171" t="n"/>
-      <c r="C18" s="166" t="n">
-        <v>1042.65</v>
-      </c>
+      <c r="C18" s="166" t="n"/>
       <c r="D18" s="167" t="n">
-        <v>969.9299999999999</v>
+        <v>382.24</v>
       </c>
       <c r="E18" s="168" t="n">
-        <v>1342.21</v>
+        <v>1732.19</v>
       </c>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
@@ -6248,7 +6254,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.173315926717876</v>
+        <v>0.23191152240805</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6289,14 +6295,12 @@
         </is>
       </c>
       <c r="B19" s="171" t="n"/>
-      <c r="C19" s="166" t="n">
-        <v>723.87</v>
-      </c>
+      <c r="C19" s="166" t="n"/>
       <c r="D19" s="167" t="n">
-        <v>1203.94</v>
+        <v>528.78</v>
       </c>
       <c r="E19" s="168" t="n">
-        <v>1118.46</v>
+        <v>1052.06</v>
       </c>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
@@ -6312,7 +6316,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.127937073283128</v>
+        <v>0.117570831076608</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6353,14 +6357,12 @@
         </is>
       </c>
       <c r="B20" s="171" t="n"/>
-      <c r="C20" s="172" t="n">
-        <v>4167.73</v>
-      </c>
+      <c r="C20" s="172" t="n"/>
       <c r="D20" s="168" t="n">
-        <v>3395.28</v>
+        <v>2313.43</v>
       </c>
       <c r="E20" s="168" t="n">
-        <v>7625.05</v>
+        <v>12696.55</v>
       </c>
       <c r="F20" s="169">
         <f>-B35</f>
@@ -6379,7 +6381,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.161308652402279</v>
+        <v>0.171970688100311</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6420,14 +6422,12 @@
         </is>
       </c>
       <c r="B21" s="171" t="n"/>
-      <c r="C21" s="166" t="n">
-        <v>2560.89</v>
-      </c>
+      <c r="C21" s="166" t="n"/>
       <c r="D21" s="167" t="n">
-        <v>1090.1</v>
+        <v>2211.06</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>2337.87</v>
+        <v>5393.66</v>
       </c>
       <c r="F21" s="169">
         <f>-B36</f>
@@ -6446,7 +6446,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.130111601586059</v>
+        <v>0.152966697937949</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6488,8 +6488,12 @@
       </c>
       <c r="B22" s="171" t="n"/>
       <c r="C22" s="172" t="n"/>
-      <c r="D22" s="168" t="n"/>
-      <c r="E22" s="168" t="n"/>
+      <c r="D22" s="168" t="n">
+        <v>8290.190000000001</v>
+      </c>
+      <c r="E22" s="168" t="n">
+        <v>39662.69915</v>
+      </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
         <v/>
@@ -6506,7 +6510,9 @@
         <f>+H22/E22</f>
         <v/>
       </c>
-      <c r="J22" s="39" t="n"/>
+      <c r="J22" s="39" t="n">
+        <v>0.191564268514993</v>
+      </c>
       <c r="K22" s="162">
         <f>E22*L22</f>
         <v/>
@@ -6546,11 +6552,13 @@
         </is>
       </c>
       <c r="B23" s="171" t="n"/>
-      <c r="C23" s="172" t="n">
-        <v>3492.43</v>
-      </c>
-      <c r="D23" s="168" t="n"/>
-      <c r="E23" s="168" t="n"/>
+      <c r="C23" s="172" t="n"/>
+      <c r="D23" s="168" t="n">
+        <v>4126.51</v>
+      </c>
+      <c r="E23" s="168" t="n">
+        <v>8732.61622</v>
+      </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
         <v/>
@@ -6567,7 +6575,9 @@
         <f>+H23/E23</f>
         <v/>
       </c>
-      <c r="J23" s="39" t="n"/>
+      <c r="J23" s="39" t="n">
+        <v>0.411717319234258</v>
+      </c>
       <c r="K23" s="162">
         <f>E23*L23</f>
         <v/>
@@ -6607,13 +6617,13 @@
         </is>
       </c>
       <c r="B24" s="173" t="n"/>
-      <c r="C24" s="174" t="n">
-        <v>247.87</v>
-      </c>
+      <c r="C24" s="174" t="n"/>
       <c r="D24" s="175" t="n">
-        <v>23.33</v>
-      </c>
-      <c r="E24" s="168" t="n"/>
+        <v>247.62</v>
+      </c>
+      <c r="E24" s="168" t="n">
+        <v>24964.47</v>
+      </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
         <v/>
@@ -6630,7 +6640,9 @@
         <f>+H24/E24</f>
         <v/>
       </c>
-      <c r="J24" s="39" t="n"/>
+      <c r="J24" s="39" t="n">
+        <v>0.199809851761323</v>
+      </c>
       <c r="K24" s="162">
         <f>E24*L24</f>
         <v/>
@@ -7029,7 +7041,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>1444.38</v>
+        <v>2289.593</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7056,7 +7068,7 @@
         </is>
       </c>
       <c r="I39" s="189" t="n">
-        <v>525.148</v>
+        <v>89.05999999999999</v>
       </c>
       <c r="J39" s="27" t="n"/>
     </row>
@@ -7089,7 +7101,7 @@
         </is>
       </c>
       <c r="I40" s="189" t="n">
-        <v>151.559</v>
+        <v>85.089</v>
       </c>
       <c r="J40" s="27" t="n"/>
     </row>
@@ -7110,7 +7122,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>254.622</v>
+        <v>117.171</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7135,7 +7147,7 @@
         </is>
       </c>
       <c r="I42" s="189" t="n">
-        <v>130.284</v>
+        <v>156.274</v>
       </c>
       <c r="J42" s="27" t="n"/>
     </row>
@@ -7156,7 +7168,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>1997</v>
+        <v>291.06</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7181,7 +7193,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>1182.893</v>
+        <v>1659.912</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7202,7 +7214,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>847.48</v>
+        <v>434.218</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7227,7 +7239,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>1155.197</v>
+        <v>812.134</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7248,7 +7260,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>1779.819</v>
+        <v>1408.026</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7282,7 +7294,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>1282</v>
+        <v>986.03</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7295,7 +7307,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>773.7180000000001</v>
+        <v>262.297</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7493,62 +7505,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-06-06</t>
+          <t>P&amp;L Build Log - Week Ending 2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\stocktake\Stocktake_2026-06-06.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\stocktake\Stocktake_2026-06-13.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_standard\OPR_Standard_WEEK_2026-06-06.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_standard\OPR_Standard_WEEK_2026-06-13.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_standard\OPR_Standard_SAT_2026-06-06.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_standard\OPR_Standard_SAT_2026-06-13.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_meat\OPR_Meat_WEEK_2026-06-06.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_meat\OPR_Meat_WEEK_2026-06-13.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\opr_meat\OPR_Meat_SAT_2026-06-06.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_meat\OPR_Meat_SAT_2026-06-13.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\waste\Waste_WEEK_2026-06-06.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\waste\Waste_WEEK_2026-06-13.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-06\waste\Waste_DAY_2026-06-06.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\waste\Waste_DAY_2026-06-13.xlsx</t>
         </is>
       </c>
     </row>
@@ -7562,273 +7574,371 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-05-30.xlsx</t>
+          <t>INFO: No previous week file found for 2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-05-30.xlsx</t>
+          <t>OK OPR std SAT: Cigarettes = 7137.91 row 13</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Beef = 9958.34 row 16</t>
+          <t>OK OPR std SAT: Produce = 39662.70 row 22</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Lamb = 964.73 row 17</t>
+          <t>OK OPR std SAT: Deli = 8732.62 row 23</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Pork = 1342.21 row 18</t>
+          <t>OK OPR std SAT: Provisions = 24964.47 row 24</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 1118.46 row 19</t>
+          <t>OK OPR meat SAT: Beef = 13218.63 row 16</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Poultry = 7625.05 row 20</t>
+          <t>OK OPR meat SAT: Lamb = 1562.31 row 17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Fish = 2337.87 row 21</t>
+          <t>OK OPR meat SAT: Pork = 1732.19 row 18</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: grocery_impulse row 30</t>
+          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 1052.06 row 19</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: grocery_edible row 31</t>
+          <t>OK OPR meat SAT: Poultry = 12696.55 row 20</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: grocery_non_food row 32</t>
+          <t>OK OPR meat SAT: Fish = 5393.66 row 21</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: baby_kids row 33</t>
+          <t>SKIP waste top-section: grocery_impulse row 30</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: personal_care row 34</t>
+          <t>SKIP waste top-section: grocery_edible row 31</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 1444.38 row 37</t>
+          <t>OK waste: Fish = 1659.91 row 44</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: meat_total row 38</t>
+          <t>SKIP waste top-section: grocery_non_food row 32</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 1182.89 row 44</t>
+          <t>SKIP waste top-section: baby_kids row 33</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OK waste: Bacon = 130.28 row 42</t>
+          <t>SKIP waste top-section: personal_care row 34</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 847.48 row 45</t>
+          <t>SKIP waste top-section: beer_wine_spirits row 35</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 1155.20 row 46</t>
+          <t>OK waste: Produce = 2289.59 row 37</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 1779.82 row 47</t>
+          <t>SKIP waste top-section: meat_total row 38</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 1282.00 row 48</t>
+          <t>OK waste: dairy = 434.22 row 45</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 773.72 row 49</t>
+          <t>OK waste: bread_cakes = 812.13 row 46</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: Beef = 525.15 row 39</t>
+          <t>OK waste: Deli = 1408.03 row 47</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: Lamb = 151.56 row 40</t>
+          <t>OK waste: Provisions = 986.03 row 48</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 254.62 row 41</t>
+          <t>OK waste: frozen = 262.30 row 49</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 1997.00 row 43</t>
+          <t>OK waste: Beef = 89.06 row 39</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 1090.10 row 21</t>
+          <t>OK waste: Lamb = 85.09 row 40</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 1203.94 row 19</t>
+          <t>OK waste: Pork = 117.17 row 41</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 6600.05 row 16</t>
+          <t>OK waste: Bacon = 156.27 row 42</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 969.93 row 18</t>
+          <t>OK waste: Poultry = 291.06 row 43</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 635.54 row 17</t>
+          <t>OK stocktake: Cigarettes = 114751.02 row 13</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 3395.28 row 20</t>
+          <t>OK stocktake: Produce = 8290.19 row 22</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 23.33 row 24</t>
+          <t>OK stocktake: Fish = 2211.06 row 21</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.17</t>
+          <t>OK stocktake: Pork = 382.24 row 18</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.26</t>
+          <t>OK stocktake: Beef = 1369.36 row 16</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.17</t>
+          <t>OK stocktake: Poultry = 2313.43 row 20</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.13</t>
+          <t>OK stocktake: Lamb = 260.86 row 17</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.16</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 528.78 row 19</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 21: 0.13</t>
+          <t>OK stocktake: Deli = 4126.51 row 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>OK stocktake: Provisions = 247.62 row 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>OK sales inc vat G4: 367581.78</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>OK sales ex vat G5: 338366.78</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>OK margin G6: 0.1741</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 13: 0.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 22: 0.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 23: 0.41</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 24: 0.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 16: 0.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 17: 0.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 18: 0.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 19: 0.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 20: 0.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 21: 0.15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Managers Report we 2026-06-20
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 13.6.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 20.6.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5714,7 +5714,7 @@
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
       <c r="G4" s="150" t="n">
-        <v>367581.78</v>
+        <v>306342.76</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -5729,7 +5729,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>338366.7843</v>
+        <v>282043.19659</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5743,7 +5743,7 @@
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
       <c r="G6" s="38" t="n">
-        <v>0.174070526992918</v>
+        <v>0.16935204414604</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5926,13 +5926,13 @@
       </c>
       <c r="B13" s="156" t="n"/>
       <c r="C13" s="157" t="n">
-        <v>123650.7399999999</v>
+        <v>114751.02</v>
       </c>
       <c r="D13" s="158" t="n">
-        <v>114751.02</v>
+        <v>127896.5799999999</v>
       </c>
       <c r="E13" s="159" t="n">
-        <v>7137.91078</v>
+        <v>6708.89439</v>
       </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
@@ -5948,7 +5948,7 @@
         <v/>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0.128699141571506</v>
+        <v>0.120741545910667</v>
       </c>
       <c r="K13" s="162">
         <f>E13*L13</f>
@@ -6109,13 +6109,13 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n">
-        <v>10799.53</v>
+        <v>1369.36</v>
       </c>
       <c r="D16" s="167" t="n">
-        <v>1369.36</v>
+        <v>9554.630000000001</v>
       </c>
       <c r="E16" s="168" t="n">
-        <v>13218.63</v>
+        <v>11111.08</v>
       </c>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
@@ -6134,7 +6134,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.195678226109665</v>
+        <v>0.203699589058849</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6176,13 +6176,13 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n">
-        <v>1065.31</v>
+        <v>260.86</v>
       </c>
       <c r="D17" s="168" t="n">
-        <v>260.86</v>
+        <v>1507.63</v>
       </c>
       <c r="E17" s="168" t="n">
-        <v>1562.31</v>
+        <v>1119.07</v>
       </c>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
@@ -6198,7 +6198,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.247975696244663</v>
+        <v>0.263373372532549</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6240,13 +6240,13 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n">
-        <v>527.65</v>
+        <v>382.24</v>
       </c>
       <c r="D18" s="167" t="n">
-        <v>382.24</v>
+        <v>1148.07</v>
       </c>
       <c r="E18" s="168" t="n">
-        <v>1732.19</v>
+        <v>1259.9</v>
       </c>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.23191152240805</v>
+        <v>0.231580077783951</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6304,13 +6304,13 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n">
-        <v>595.9400000000001</v>
+        <v>528.78</v>
       </c>
       <c r="D19" s="167" t="n">
-        <v>528.78</v>
+        <v>802.55</v>
       </c>
       <c r="E19" s="168" t="n">
-        <v>1052.06</v>
+        <v>762.9699999999999</v>
       </c>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
@@ -6326,7 +6326,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.117570831076608</v>
+        <v>0.109901758987371</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6368,13 +6368,13 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n">
-        <v>1953.62</v>
+        <v>2313.43</v>
       </c>
       <c r="D20" s="168" t="n">
-        <v>2313.43</v>
+        <v>3571.79</v>
       </c>
       <c r="E20" s="168" t="n">
-        <v>12696.55</v>
+        <v>10565.04</v>
       </c>
       <c r="F20" s="169">
         <f>-B35</f>
@@ -6393,7 +6393,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.171970688100311</v>
+        <v>0.167681863958868</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6435,13 +6435,13 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n">
-        <v>2243.06</v>
+        <v>2211.06</v>
       </c>
       <c r="D21" s="167" t="n">
-        <v>2211.06</v>
+        <v>2138.81</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>5393.66</v>
+        <v>4645.86</v>
       </c>
       <c r="F21" s="169">
         <f>-B36</f>
@@ -6460,7 +6460,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.152966697937949</v>
+        <v>0.178751410933605</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6502,13 +6502,11 @@
       </c>
       <c r="B22" s="171" t="n"/>
       <c r="C22" s="172" t="n">
-        <v>9759.909999999991</v>
-      </c>
-      <c r="D22" s="168" t="n">
         <v>8290.190000000001</v>
       </c>
+      <c r="D22" s="168" t="n"/>
       <c r="E22" s="168" t="n">
-        <v>39662.69915</v>
+        <v>33320.80816</v>
       </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
@@ -6527,7 +6525,7 @@
         <v/>
       </c>
       <c r="J22" s="39" t="n">
-        <v>0.191564268514993</v>
+        <v>0.190189436269663</v>
       </c>
       <c r="K22" s="162">
         <f>E22*L22</f>
@@ -6569,13 +6567,13 @@
       </c>
       <c r="B23" s="171" t="n"/>
       <c r="C23" s="172" t="n">
-        <v>4075.56</v>
+        <v>4126.51</v>
       </c>
       <c r="D23" s="168" t="n">
-        <v>4126.51</v>
+        <v>3609.59</v>
       </c>
       <c r="E23" s="168" t="n">
-        <v>8732.61622</v>
+        <v>7714.70862</v>
       </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
@@ -6594,7 +6592,7 @@
         <v/>
       </c>
       <c r="J23" s="39" t="n">
-        <v>0.411717319234258</v>
+        <v>0.398113528492538</v>
       </c>
       <c r="K23" s="162">
         <f>E23*L23</f>
@@ -6636,13 +6634,13 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n">
-        <v>49.67</v>
+        <v>247.62</v>
       </c>
       <c r="D24" s="175" t="n">
-        <v>247.62</v>
+        <v>210.9</v>
       </c>
       <c r="E24" s="168" t="n">
-        <v>24964.47</v>
+        <v>21563.35</v>
       </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
@@ -6661,7 +6659,7 @@
         <v/>
       </c>
       <c r="J24" s="39" t="n">
-        <v>0.199809851761323</v>
+        <v>0.198677533871129</v>
       </c>
       <c r="K24" s="162">
         <f>E24*L24</f>
@@ -7061,7 +7059,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>2289.593</v>
+        <v>1684.83</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7088,7 +7086,7 @@
         </is>
       </c>
       <c r="I39" s="189" t="n">
-        <v>89.05999999999999</v>
+        <v>69.05</v>
       </c>
       <c r="J39" s="27" t="n"/>
     </row>
@@ -7121,7 +7119,7 @@
         </is>
       </c>
       <c r="I40" s="189" t="n">
-        <v>85.089</v>
+        <v>38.36</v>
       </c>
       <c r="J40" s="27" t="n"/>
     </row>
@@ -7142,7 +7140,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>117.171</v>
+        <v>41.28</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7167,7 +7165,7 @@
         </is>
       </c>
       <c r="I42" s="189" t="n">
-        <v>156.274</v>
+        <v>5.4</v>
       </c>
       <c r="J42" s="27" t="n"/>
     </row>
@@ -7188,7 +7186,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>291.06</v>
+        <v>48.27</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7213,7 +7211,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>1659.912</v>
+        <v>1291.08</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7234,7 +7232,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>434.218</v>
+        <v>377.28</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7259,7 +7257,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>812.134</v>
+        <v>446.38</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7280,7 +7278,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>1408.026</v>
+        <v>484.54</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7314,7 +7312,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>986.03</v>
+        <v>701.9400000000001</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7327,7 +7325,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>262.297</v>
+        <v>219.25</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7525,62 +7523,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-06-13</t>
+          <t>P&amp;L Build Log - Week Ending 2026-06-20</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\stocktake\Stocktake_2026-06-13.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\stocktake\Stocktake_2026-06-20.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_standard\OPR_Standard_WEEK_2026-06-13.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_standard\OPR_Standard_WEEK_2026-06-20.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_standard\OPR_Standard_SAT_2026-06-13.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_standard\OPR_Standard_SAT_2026-06-20.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_meat\OPR_Meat_WEEK_2026-06-13.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_meat\OPR_Meat_WEEK_2026-06-20.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\opr_meat\OPR_Meat_SAT_2026-06-13.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_meat\OPR_Meat_SAT_2026-06-20.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\waste\Waste_WEEK_2026-06-13.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\waste\Waste_WEEK_2026-06-20.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-13\waste\Waste_DAY_2026-06-13.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\waste\Waste_DAY_2026-06-20.xlsx</t>
         </is>
       </c>
     </row>
@@ -7594,84 +7592,84 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-06-06-v2.xlsx</t>
+          <t>INFO: Previous week file: Managers_Report_we_2026-06-13-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-06-06-v2.xlsx</t>
+          <t>OK opening stock from Managers_Report_we_2026-06-13-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Cigarettes = 7137.91 row 13</t>
+          <t>OK OPR std SAT: Cigarettes = 6708.89 row 13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Produce = 39662.70 row 22</t>
+          <t>OK OPR std SAT: Produce = 33320.81 row 22</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Deli = 8732.62 row 23</t>
+          <t>OK OPR std SAT: Deli = 7714.71 row 23</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Provisions = 24964.47 row 24</t>
+          <t>OK OPR std SAT: Provisions = 21563.35 row 24</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Beef = 13218.63 row 16</t>
+          <t>OK OPR meat SAT: Beef = 11111.08 row 16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Lamb = 1562.31 row 17</t>
+          <t>OK OPR meat SAT: Lamb = 1119.07 row 17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Pork = 1732.19 row 18</t>
+          <t>OK OPR meat SAT: Pork = 1259.90 row 18</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 1052.06 row 19</t>
+          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 762.97 row 19</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Poultry = 12696.55 row 20</t>
+          <t>OK OPR meat SAT: Poultry = 10565.04 row 20</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Fish = 5393.66 row 21</t>
+          <t>OK OPR meat SAT: Fish = 4645.86 row 21</t>
         </is>
       </c>
     </row>
@@ -7692,7 +7690,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 1659.91 row 44</t>
+          <t>OK waste: Fish = 1291.08 row 44</t>
         </is>
       </c>
     </row>
@@ -7713,259 +7711,252 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: personal_care row 34</t>
+          <t>SKIP waste top-section: beer_wine_spirits row 35</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: beer_wine_spirits row 35</t>
+          <t>OK waste: Produce = 1684.83 row 37</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 2289.59 row 37</t>
+          <t>SKIP waste top-section: meat_total row 38</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: meat_total row 38</t>
+          <t>OK waste: dairy = 377.28 row 45</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 434.22 row 45</t>
+          <t>OK waste: bread_cakes = 446.38 row 46</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 812.13 row 46</t>
+          <t>OK waste: Deli = 484.54 row 47</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 1408.03 row 47</t>
+          <t>OK waste: Provisions = 701.94 row 48</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 986.03 row 48</t>
+          <t>OK waste: frozen = 219.25 row 49</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 262.30 row 49</t>
+          <t>OK waste: Beef = 69.05 row 39</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK waste: Beef = 89.06 row 39</t>
+          <t>OK waste: Lamb = 38.36 row 40</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK waste: Lamb = 85.09 row 40</t>
+          <t>OK waste: Pork = 41.28 row 41</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 117.17 row 41</t>
+          <t>OK waste: Bacon = 5.40 row 42</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK waste: Bacon = 156.27 row 42</t>
+          <t>OK waste: Poultry = 48.27 row 43</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 291.06 row 43</t>
+          <t>SKIP waste top-section: personal_care row 34</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK stocktake: Cigarettes = 114751.02 row 13</t>
+          <t>OK stocktake: Cigarettes = 127896.58 row 13</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK stocktake: Produce = 8290.19 row 22</t>
+          <t>OK stocktake: Fish = 2138.81 row 21</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 2211.06 row 21</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 802.55 row 19</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 382.24 row 18</t>
+          <t>OK stocktake: Beef = 9554.63 row 16</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 1369.36 row 16</t>
+          <t>OK stocktake: Lamb = 1507.63 row 17</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 2313.43 row 20</t>
+          <t>OK stocktake: Pork = 1148.07 row 18</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 260.86 row 17</t>
+          <t>OK stocktake: Poultry = 3571.79 row 20</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 528.78 row 19</t>
+          <t>OK stocktake: Deli = 3609.59 row 23</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK stocktake: Deli = 4126.51 row 23</t>
+          <t>OK stocktake: Provisions = 210.90 row 24</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 247.62 row 24</t>
+          <t>OK sales inc vat G4: 306342.76</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 367581.78</t>
+          <t>OK sales ex vat G5: 282043.20</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 338366.78</t>
+          <t>OK margin G6: 0.1694</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1741</t>
+          <t>OK scan margin std row 13: 0.12</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.13</t>
+          <t>OK scan margin std row 22: 0.19</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.19</t>
+          <t>OK scan margin std row 23: 0.40</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OK scan margin std row 23: 0.41</t>
+          <t>OK scan margin std row 24: 0.20</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>OK scan margin std row 24: 0.20</t>
+          <t>OK scan margin meat row 16: 0.20</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.20</t>
+          <t>OK scan margin meat row 17: 0.26</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.25</t>
+          <t>OK scan margin meat row 18: 0.23</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.23</t>
+          <t>OK scan margin meat row 19: 0.11</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.12</t>
+          <t>OK scan margin meat row 20: 0.17</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.17</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>OK scan margin meat row 21: 0.15</t>
+          <t>OK scan margin meat row 21: 0.18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Managers Report we 2026-06-27
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 20.6.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 27.6.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5714,7 +5714,7 @@
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
       <c r="G4" s="150" t="n">
-        <v>301811.98</v>
+        <v>394761.22</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -5729,7 +5729,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>274726.07099</v>
+        <v>361766.90862</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5743,7 +5743,7 @@
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
       <c r="G6" s="38" t="n">
-        <v>0.177878545796183</v>
+        <v>0.175879837165633</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5925,10 +5925,14 @@
         </is>
       </c>
       <c r="B13" s="156" t="n"/>
-      <c r="C13" s="157" t="n"/>
-      <c r="D13" s="158" t="n"/>
+      <c r="C13" s="157" t="n">
+        <v>127896.5799999999</v>
+      </c>
+      <c r="D13" s="158" t="n">
+        <v>131469.13</v>
+      </c>
       <c r="E13" s="159" t="n">
-        <v>10567.72368</v>
+        <v>7652.95136</v>
       </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
@@ -5944,7 +5948,7 @@
         <v/>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0.0939446876226423</v>
+        <v>0.129586996355874</v>
       </c>
       <c r="K13" s="162">
         <f>E13*L13</f>
@@ -6105,13 +6109,13 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n">
-        <v>7116.87</v>
+        <v>9554.630000000001</v>
       </c>
       <c r="D16" s="167" t="n">
-        <v>6390.379999999999</v>
+        <v>11161.92</v>
       </c>
       <c r="E16" s="168" t="n">
-        <v>11743.72</v>
+        <v>13832.32</v>
       </c>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
@@ -6130,7 +6134,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.17537033495349</v>
+        <v>0.194777774082728</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6172,13 +6176,13 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n">
-        <v>665.49</v>
+        <v>1507.63</v>
       </c>
       <c r="D17" s="168" t="n">
-        <v>455.47</v>
+        <v>1182.86</v>
       </c>
       <c r="E17" s="168" t="n">
-        <v>1037.45</v>
+        <v>1490.55</v>
       </c>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
@@ -6194,7 +6198,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.237793522579401</v>
+        <v>0.241053872731542</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6236,13 +6240,13 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n">
-        <v>484.08</v>
+        <v>1148.07</v>
       </c>
       <c r="D18" s="167" t="n">
-        <v>669.78</v>
+        <v>1209.33</v>
       </c>
       <c r="E18" s="168" t="n">
-        <v>1128.82</v>
+        <v>1619.89</v>
       </c>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
@@ -6258,7 +6262,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.182388077815772</v>
+        <v>0.207649920673626</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6300,13 +6304,13 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n">
-        <v>1174.44</v>
+        <v>802.55</v>
       </c>
       <c r="D19" s="167" t="n">
-        <v>758.1700000000001</v>
+        <v>512.42</v>
       </c>
       <c r="E19" s="168" t="n">
-        <v>1082.51</v>
+        <v>876.64</v>
       </c>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
@@ -6322,7 +6326,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.119882297340407</v>
+        <v>0.112630328255635</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6364,13 +6368,13 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n">
-        <v>2754.95</v>
+        <v>3571.79</v>
       </c>
       <c r="D20" s="168" t="n">
-        <v>3336.37</v>
+        <v>2228</v>
       </c>
       <c r="E20" s="168" t="n">
-        <v>8092.91</v>
+        <v>13289.83</v>
       </c>
       <c r="F20" s="169">
         <f>-B35</f>
@@ -6389,7 +6393,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.161722302608085</v>
+        <v>0.167672840811357</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6431,13 +6435,13 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n">
-        <v>1105.76</v>
+        <v>2138.81</v>
       </c>
       <c r="D21" s="167" t="n">
-        <v>1063.48</v>
+        <v>1990.5</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>2271.51</v>
+        <v>5599.62</v>
       </c>
       <c r="F21" s="169">
         <f>-B36</f>
@@ -6456,7 +6460,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.177538245484281</v>
+        <v>0.177858572545994</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6497,12 +6501,12 @@
         </is>
       </c>
       <c r="B22" s="171" t="n"/>
-      <c r="C22" s="172" t="n">
-        <v>8152.47</v>
-      </c>
-      <c r="D22" s="168" t="n"/>
+      <c r="C22" s="172" t="n"/>
+      <c r="D22" s="168" t="n">
+        <v>11162.64</v>
+      </c>
       <c r="E22" s="168" t="n">
-        <v>26297.1639</v>
+        <v>42313.26172</v>
       </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
@@ -6521,7 +6525,7 @@
         <v/>
       </c>
       <c r="J22" s="39" t="n">
-        <v>0.1966209432189</v>
+        <v>0.190597038426562</v>
       </c>
       <c r="K22" s="162">
         <f>E22*L22</f>
@@ -6562,10 +6566,14 @@
         </is>
       </c>
       <c r="B23" s="171" t="n"/>
-      <c r="C23" s="172" t="n"/>
-      <c r="D23" s="168" t="n"/>
+      <c r="C23" s="172" t="n">
+        <v>3609.59</v>
+      </c>
+      <c r="D23" s="168" t="n">
+        <v>3880.07</v>
+      </c>
       <c r="E23" s="168" t="n">
-        <v>10599.52164</v>
+        <v>10663.41415</v>
       </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
@@ -6584,7 +6592,7 @@
         <v/>
       </c>
       <c r="J23" s="39" t="n">
-        <v>0.717072689289885</v>
+        <v>0.393789152417005</v>
       </c>
       <c r="K23" s="162">
         <f>E23*L23</f>
@@ -6626,13 +6634,13 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n">
-        <v>24.18</v>
+        <v>210.9</v>
       </c>
       <c r="D24" s="175" t="n">
-        <v>17.09</v>
+        <v>25129.61</v>
       </c>
       <c r="E24" s="168" t="n">
-        <v>18004.6</v>
+        <v>26098.97</v>
       </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
@@ -6651,7 +6659,7 @@
         <v/>
       </c>
       <c r="J24" s="39" t="n">
-        <v>0.217554569387823</v>
+        <v>0.194783830932792</v>
       </c>
       <c r="K24" s="162">
         <f>E24*L24</f>
@@ -7051,7 +7059,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>730.02</v>
+        <v>888.48</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7077,7 +7085,9 @@
           <t>- Beef</t>
         </is>
       </c>
-      <c r="I39" s="189" t="n"/>
+      <c r="I39" s="189" t="n">
+        <v>64.48999999999999</v>
+      </c>
       <c r="J39" s="27" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" thickBot="1">
@@ -7108,7 +7118,9 @@
           <t>- Lamb</t>
         </is>
       </c>
-      <c r="I40" s="189" t="n"/>
+      <c r="I40" s="189" t="n">
+        <v>38.36</v>
+      </c>
       <c r="J40" s="27" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -7128,7 +7140,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>14.7</v>
+        <v>6.96</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7153,7 +7165,7 @@
         </is>
       </c>
       <c r="I42" s="189" t="n">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="J42" s="27" t="n"/>
     </row>
@@ -7174,7 +7186,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>191.24</v>
+        <v>30.29</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7199,7 +7211,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>310.35</v>
+        <v>522.7</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7220,7 +7232,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>769.73</v>
+        <v>403.77</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7245,7 +7257,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>406.21</v>
+        <v>390.75</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7266,7 +7278,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>481.83</v>
+        <v>255.83</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7300,7 +7312,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>713.9300000000001</v>
+        <v>1000.74</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7313,7 +7325,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>2.49</v>
+        <v>96.81</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7511,62 +7523,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-06-20</t>
+          <t>P&amp;L Build Log - Week Ending 2026-06-27</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\stocktake\Stocktake_2026-06-20.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\stocktake\Stocktake_2026-06-27.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_standard\OPR_Standard_WEEK_2026-06-20.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_standard\OPR_Standard_WEEK_2026-06-27.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_standard\OPR_Standard_SAT_2026-06-20.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_standard\OPR_Standard_SAT_2026-06-27.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_meat\OPR_Meat_WEEK_2026-06-20.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_meat\OPR_Meat_WEEK_2026-06-27.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\opr_meat\OPR_Meat_SAT_2026-06-20.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_meat\OPR_Meat_SAT_2026-06-27.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\waste\Waste_WEEK_2026-06-20.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\waste\Waste_WEEK_2026-06-27.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-20\waste\Waste_DAY_2026-06-20.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\waste\Waste_DAY_2026-06-27.xlsx</t>
         </is>
       </c>
     </row>
@@ -7580,84 +7592,84 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-06-13-v2.xlsx</t>
+          <t>INFO: Previous week file: Managers_Report_we_2026-06-20-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-06-13-v2.xlsx</t>
+          <t>OK opening stock from Managers_Report_we_2026-06-20-v3.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Cigarettes = 10567.72 row 13</t>
+          <t>OK OPR std SAT: Cigarettes = 7652.95 row 13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Produce = 26297.16 row 22</t>
+          <t>OK OPR std SAT: Produce = 42313.26 row 22</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Deli = 10599.52 row 23</t>
+          <t>OK OPR std SAT: Deli = 10663.41 row 23</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Provisions = 18004.60 row 24</t>
+          <t>OK OPR std SAT: Provisions = 26098.97 row 24</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Beef = 11743.72 row 16</t>
+          <t>OK OPR meat SAT: Beef = 13832.32 row 16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Lamb = 1037.45 row 17</t>
+          <t>OK OPR meat SAT: Lamb = 1490.55 row 17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Pork = 1128.82 row 18</t>
+          <t>OK OPR meat SAT: Pork = 1619.89 row 18</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 1082.51 row 19</t>
+          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 876.64 row 19</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Poultry = 8092.91 row 20</t>
+          <t>OK OPR meat SAT: Poultry = 13289.83 row 20</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Fish = 2271.51 row 21</t>
+          <t>OK OPR meat SAT: Fish = 5599.62 row 21</t>
         </is>
       </c>
     </row>
@@ -7685,222 +7697,271 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: personal_care row 34</t>
+          <t>SKIP waste top-section: baby_kids row 33</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 730.02 row 37</t>
+          <t>SKIP waste top-section: personal_care row 34</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: meat_total row 38</t>
+          <t>OK waste: Produce = 888.48 row 37</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 769.73 row 45</t>
+          <t>SKIP waste top-section: meat_total row 38</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 406.21 row 46</t>
+          <t>OK waste: dairy = 403.77 row 45</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 481.83 row 47</t>
+          <t>OK waste: bread_cakes = 390.75 row 46</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 713.93 row 48</t>
+          <t>OK waste: Deli = 255.83 row 47</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 2.49 row 49</t>
+          <t>OK waste: Provisions = 1000.74 row 48</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 14.70 row 41</t>
+          <t>OK waste: frozen = 96.81 row 49</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: Bacon = 0.00 row 42</t>
+          <t>OK waste: Beef = 64.49 row 39</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 191.24 row 43</t>
+          <t>OK waste: Lamb = 38.36 row 40</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 310.35 row 44</t>
+          <t>OK waste: Pork = 6.96 row 41</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 1063.48 row 21</t>
+          <t>OK waste: Bacon = 5.40 row 42</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 758.17 row 19</t>
+          <t>OK waste: Poultry = 30.29 row 43</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 6390.38 row 16</t>
+          <t>OK waste: Fish = 522.70 row 44</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 455.47 row 17</t>
+          <t>SKIP waste top-section: beer_wine_spirits row 35</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 669.78 row 18</t>
+          <t>OK stocktake: Cigarettes = 131469.13 row 13</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 3336.37 row 20</t>
+          <t>OK stocktake: Produce = 11162.64 row 22</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 17.09 row 24</t>
+          <t>OK stocktake: Fish = 1990.50 row 21</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 301811.98</t>
+          <t>OK stocktake: Beef = 11161.92 row 16</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 274726.07</t>
+          <t>OK stocktake: Pork = 1209.33 row 18</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1779</t>
+          <t>OK stocktake: Lamb = 1182.86 row 17</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.09</t>
+          <t>OK stocktake: Poultry = 2228.00 row 20</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.20</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 512.42 row 19</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK scan margin std row 23: 0.72</t>
+          <t>OK stocktake: Deli = 3880.07 row 23</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK scan margin std row 24: 0.22</t>
+          <t>OK stocktake: Provisions = 25129.61 row 24</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.18</t>
+          <t>OK sales inc vat G4: 394761.22</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.24</t>
+          <t>OK sales ex vat G5: 361766.91</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.18</t>
+          <t>OK margin G6: 0.1759</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.12</t>
+          <t>OK scan margin std row 13: 0.13</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.16</t>
+          <t>OK scan margin std row 22: 0.19</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 23: 0.39</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 24: 0.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 16: 0.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 17: 0.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 18: 0.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 19: 0.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 20: 0.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>OK scan margin meat row 21: 0.18</t>
         </is>

</xml_diff>

<commit_message>
Managers Report we 2026-07-04
</commit_message>
<xml_diff>
--- a/data/managers_report_latest.xlsx
+++ b/data/managers_report_latest.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="16.01.24" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="TEMPLATE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="we 27.6.26" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="we 4.7.26" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -5714,7 +5714,7 @@
       <c r="E4" s="149" t="n"/>
       <c r="F4" s="81" t="n"/>
       <c r="G4" s="150" t="n">
-        <v>394761.22</v>
+        <v>374316.37</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -5729,7 +5729,7 @@
       <c r="E5" s="149" t="n"/>
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="150" t="n">
-        <v>361766.90862</v>
+        <v>344109.32277</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -5743,7 +5743,7 @@
       <c r="E6" s="151" t="n"/>
       <c r="F6" s="82" t="n"/>
       <c r="G6" s="38" t="n">
-        <v>0.175879837165633</v>
+        <v>0.173147272908453</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -5926,13 +5926,13 @@
       </c>
       <c r="B13" s="156" t="n"/>
       <c r="C13" s="157" t="n">
-        <v>127896.5799999999</v>
+        <v>131469.13</v>
       </c>
       <c r="D13" s="158" t="n">
-        <v>131469.13</v>
+        <v>141369.1799999999</v>
       </c>
       <c r="E13" s="159" t="n">
-        <v>7652.95136</v>
+        <v>7811.79689</v>
       </c>
       <c r="F13" s="160" t="n"/>
       <c r="G13" s="157">
@@ -5948,7 +5948,7 @@
         <v/>
       </c>
       <c r="J13" s="39" t="n">
-        <v>0.129586996355874</v>
+        <v>0.1230964582849</v>
       </c>
       <c r="K13" s="162">
         <f>E13*L13</f>
@@ -6109,13 +6109,13 @@
       </c>
       <c r="B16" s="165" t="n"/>
       <c r="C16" s="166" t="n">
-        <v>9554.630000000001</v>
+        <v>11161.92</v>
       </c>
       <c r="D16" s="167" t="n">
-        <v>11161.92</v>
+        <v>12611.55</v>
       </c>
       <c r="E16" s="168" t="n">
-        <v>13832.32</v>
+        <v>12820.81</v>
       </c>
       <c r="F16" s="169">
         <f>-B34+D30+D33</f>
@@ -6134,7 +6134,7 @@
         <v/>
       </c>
       <c r="J16" s="39" t="n">
-        <v>0.194777774082728</v>
+        <v>0.195561323348525</v>
       </c>
       <c r="K16" s="162">
         <f>E16*L16</f>
@@ -6176,13 +6176,13 @@
       </c>
       <c r="B17" s="171" t="n"/>
       <c r="C17" s="172" t="n">
-        <v>1507.63</v>
+        <v>1182.86</v>
       </c>
       <c r="D17" s="168" t="n">
-        <v>1182.86</v>
+        <v>1334.15</v>
       </c>
       <c r="E17" s="168" t="n">
-        <v>1490.55</v>
+        <v>1327.74</v>
       </c>
       <c r="F17" s="169" t="n"/>
       <c r="G17" s="157">
@@ -6198,7 +6198,7 @@
         <v/>
       </c>
       <c r="J17" s="39" t="n">
-        <v>0.241053872731542</v>
+        <v>0.240027851838462</v>
       </c>
       <c r="K17" s="162">
         <f>E17*L17</f>
@@ -6240,13 +6240,13 @@
       </c>
       <c r="B18" s="171" t="n"/>
       <c r="C18" s="166" t="n">
-        <v>1148.07</v>
+        <v>1209.33</v>
       </c>
       <c r="D18" s="167" t="n">
-        <v>1209.33</v>
+        <v>1244.26</v>
       </c>
       <c r="E18" s="168" t="n">
-        <v>1619.89</v>
+        <v>1766.48</v>
       </c>
       <c r="F18" s="169" t="n"/>
       <c r="G18" s="157">
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="J18" s="39" t="n">
-        <v>0.207649920673626</v>
+        <v>0.207239697024591</v>
       </c>
       <c r="K18" s="162">
         <f>E18*L18</f>
@@ -6304,13 +6304,13 @@
       </c>
       <c r="B19" s="171" t="n"/>
       <c r="C19" s="166" t="n">
-        <v>802.55</v>
+        <v>512.42</v>
       </c>
       <c r="D19" s="167" t="n">
-        <v>512.42</v>
+        <v>379.27</v>
       </c>
       <c r="E19" s="168" t="n">
-        <v>876.64</v>
+        <v>1033.86</v>
       </c>
       <c r="F19" s="169" t="n"/>
       <c r="G19" s="157">
@@ -6326,7 +6326,7 @@
         <v/>
       </c>
       <c r="J19" s="39" t="n">
-        <v>0.112630328255635</v>
+        <v>0.082527414330218</v>
       </c>
       <c r="K19" s="162">
         <f>E19*L19</f>
@@ -6368,13 +6368,13 @@
       </c>
       <c r="B20" s="171" t="n"/>
       <c r="C20" s="172" t="n">
-        <v>3571.79</v>
+        <v>2228</v>
       </c>
       <c r="D20" s="168" t="n">
-        <v>2228</v>
+        <v>3023.56</v>
       </c>
       <c r="E20" s="168" t="n">
-        <v>13289.83</v>
+        <v>13032.06</v>
       </c>
       <c r="F20" s="169">
         <f>-B35</f>
@@ -6393,7 +6393,7 @@
         <v/>
       </c>
       <c r="J20" s="39" t="n">
-        <v>0.167672840811357</v>
+        <v>0.167918212469863</v>
       </c>
       <c r="K20" s="162">
         <f>E20*L20</f>
@@ -6435,13 +6435,13 @@
       </c>
       <c r="B21" s="171" t="n"/>
       <c r="C21" s="166" t="n">
-        <v>2138.81</v>
+        <v>1990.5</v>
       </c>
       <c r="D21" s="167" t="n">
-        <v>1990.5</v>
+        <v>2177.42</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>5599.62</v>
+        <v>5366.7</v>
       </c>
       <c r="F21" s="169">
         <f>-B36</f>
@@ -6460,7 +6460,7 @@
         <v/>
       </c>
       <c r="J21" s="39" t="n">
-        <v>0.177858572545994</v>
+        <v>0.177937572437438</v>
       </c>
       <c r="K21" s="162">
         <f>E21*L21</f>
@@ -6501,12 +6501,14 @@
         </is>
       </c>
       <c r="B22" s="171" t="n"/>
-      <c r="C22" s="172" t="n"/>
+      <c r="C22" s="172" t="n">
+        <v>11162.64</v>
+      </c>
       <c r="D22" s="168" t="n">
-        <v>11162.64</v>
+        <v>11832.09</v>
       </c>
       <c r="E22" s="168" t="n">
-        <v>42313.26172</v>
+        <v>40320.64575</v>
       </c>
       <c r="F22" s="169">
         <f>-B29-B30</f>
@@ -6525,7 +6527,7 @@
         <v/>
       </c>
       <c r="J22" s="39" t="n">
-        <v>0.190597038426562</v>
+        <v>0.187600911624785</v>
       </c>
       <c r="K22" s="162">
         <f>E22*L22</f>
@@ -6567,13 +6569,13 @@
       </c>
       <c r="B23" s="171" t="n"/>
       <c r="C23" s="172" t="n">
-        <v>3609.59</v>
+        <v>3880.07</v>
       </c>
       <c r="D23" s="168" t="n">
-        <v>3880.07</v>
+        <v>3163.7</v>
       </c>
       <c r="E23" s="168" t="n">
-        <v>10663.41415</v>
+        <v>10246.36926</v>
       </c>
       <c r="F23" s="169">
         <f>D29+D32+D31+D34+D35+D36+D37</f>
@@ -6592,7 +6594,7 @@
         <v/>
       </c>
       <c r="J23" s="39" t="n">
-        <v>0.393789152417005</v>
+        <v>0.399865901377831</v>
       </c>
       <c r="K23" s="162">
         <f>E23*L23</f>
@@ -6634,13 +6636,13 @@
       </c>
       <c r="B24" s="173" t="n"/>
       <c r="C24" s="174" t="n">
-        <v>210.9</v>
+        <v>25129.61</v>
       </c>
       <c r="D24" s="175" t="n">
-        <v>25129.61</v>
+        <v>319.23</v>
       </c>
       <c r="E24" s="168" t="n">
-        <v>26098.97</v>
+        <v>24479.17</v>
       </c>
       <c r="F24" s="169">
         <f>-B33-B37</f>
@@ -6659,7 +6661,7 @@
         <v/>
       </c>
       <c r="J24" s="39" t="n">
-        <v>0.194783830932792</v>
+        <v>0.190378445020807</v>
       </c>
       <c r="K24" s="162">
         <f>E24*L24</f>
@@ -7059,7 +7061,7 @@
         </is>
       </c>
       <c r="I37" s="189" t="n">
-        <v>888.48</v>
+        <v>707.3199999999999</v>
       </c>
       <c r="J37" s="27" t="n"/>
     </row>
@@ -7086,7 +7088,7 @@
         </is>
       </c>
       <c r="I39" s="189" t="n">
-        <v>64.48999999999999</v>
+        <v>0</v>
       </c>
       <c r="J39" s="27" t="n"/>
     </row>
@@ -7119,7 +7121,7 @@
         </is>
       </c>
       <c r="I40" s="189" t="n">
-        <v>38.36</v>
+        <v>0</v>
       </c>
       <c r="J40" s="27" t="n"/>
     </row>
@@ -7140,7 +7142,7 @@
         </is>
       </c>
       <c r="I41" s="189" t="n">
-        <v>6.96</v>
+        <v>0</v>
       </c>
       <c r="J41" s="27" t="n"/>
     </row>
@@ -7165,7 +7167,7 @@
         </is>
       </c>
       <c r="I42" s="189" t="n">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="J42" s="27" t="n"/>
     </row>
@@ -7186,7 +7188,7 @@
         </is>
       </c>
       <c r="I43" s="189" t="n">
-        <v>30.29</v>
+        <v>13.1</v>
       </c>
       <c r="J43" s="27" t="n"/>
     </row>
@@ -7211,7 +7213,7 @@
         </is>
       </c>
       <c r="I44" s="189" t="n">
-        <v>522.7</v>
+        <v>439.01</v>
       </c>
       <c r="J44" s="27" t="n"/>
     </row>
@@ -7232,7 +7234,7 @@
         </is>
       </c>
       <c r="I45" s="189" t="n">
-        <v>403.77</v>
+        <v>356.42</v>
       </c>
       <c r="J45" s="27" t="n"/>
     </row>
@@ -7257,7 +7259,7 @@
         </is>
       </c>
       <c r="I46" s="189" t="n">
-        <v>390.75</v>
+        <v>362.86</v>
       </c>
       <c r="J46" s="27" t="n"/>
     </row>
@@ -7278,7 +7280,7 @@
         </is>
       </c>
       <c r="I47" s="189" t="n">
-        <v>255.83</v>
+        <v>241.38</v>
       </c>
       <c r="J47" s="27" t="n"/>
     </row>
@@ -7312,7 +7314,7 @@
         </is>
       </c>
       <c r="I48" s="189" t="n">
-        <v>1000.74</v>
+        <v>1195.74</v>
       </c>
       <c r="J48" s="27" t="n"/>
     </row>
@@ -7325,7 +7327,7 @@
         </is>
       </c>
       <c r="I49" s="189" t="n">
-        <v>96.81</v>
+        <v>10.49</v>
       </c>
       <c r="J49" s="27" t="n"/>
     </row>
@@ -7523,62 +7525,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>P&amp;L Build Log - Week Ending 2026-06-27</t>
+          <t>P&amp;L Build Log - Week Ending 2026-07-04</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\stocktake\Stocktake_2026-06-27.xlsx</t>
+          <t>Downloaded STOCKTAKE: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-07-04\stocktake\Stocktake_2026-07-04.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_standard\OPR_Standard_WEEK_2026-06-27.xlsx</t>
+          <t>Downloaded OPR_STANDARD_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-07-04\opr_standard\OPR_Standard_WEEK_2026-07-04.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_standard\OPR_Standard_SAT_2026-06-27.xlsx</t>
+          <t>Downloaded OPR_STANDARD_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-07-04\opr_standard\OPR_Standard_SAT_2026-07-04.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_meat\OPR_Meat_WEEK_2026-06-27.xlsx</t>
+          <t>Downloaded OPR_MEAT_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-07-04\opr_meat\OPR_Meat_WEEK_2026-07-04.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\opr_meat\OPR_Meat_SAT_2026-06-27.xlsx</t>
+          <t>Downloaded OPR_MEAT_SAT: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-07-04\opr_meat\OPR_Meat_SAT_2026-07-04.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\waste\Waste_WEEK_2026-06-27.xlsx</t>
+          <t>Downloaded WASTE_WEEK: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-07-04\waste\Waste_WEEK_2026-07-04.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-06-27\waste\Waste_DAY_2026-06-27.xlsx</t>
+          <t>Downloaded WASTE_DAY: C:\Users\halpi\OneDrive\Desktop\PNL\exports\2026-07-04\waste\Waste_DAY_2026-07-04.xlsx</t>
         </is>
       </c>
     </row>
@@ -7592,376 +7594,446 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INFO: Previous week file: Managers_Report_we_2026-06-20-v3.xlsx</t>
+          <t>INFO: Previous week file: Managers_Report_we_2026-06-27-v2.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OK opening stock from Managers_Report_we_2026-06-20-v3.xlsx</t>
+          <t>OK opening stock from Managers_Report_we_2026-06-27-v2.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Cigarettes = 7652.95 row 13</t>
+          <t>MISS OPR std SAT: Grocery Impulse</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Produce = 42313.26 row 22</t>
+          <t>MISS OPR std SAT: Grocery Edible</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Deli = 10663.41 row 23</t>
+          <t>MISS OPR std SAT: Grocery Non Food</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>OK OPR std SAT: Provisions = 26098.97 row 24</t>
+          <t>MISS OPR std SAT: Baby &amp; Kids</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Beef = 13832.32 row 16</t>
+          <t>MISS OPR std SAT: Personal Care</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Lamb = 1490.55 row 17</t>
+          <t>MISS OPR std SAT: Beer Wine Spirits</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Pork = 1619.89 row 18</t>
+          <t>OK OPR std SAT: Cigarettes = 7811.80 row 13</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 876.64 row 19</t>
+          <t>OK OPR std SAT: Produce = 40320.65 row 22</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Poultry = 13289.83 row 20</t>
+          <t>MISS OPR std SAT: Dairy</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OK OPR meat SAT: Fish = 5599.62 row 21</t>
+          <t>MISS OPR std SAT: Bread &amp; Cakes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: grocery_impulse row 30</t>
+          <t>OK OPR std SAT: Deli = 10246.37 row 23</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: grocery_edible row 31</t>
+          <t>OK OPR std SAT: Provisions = 24479.17 row 24</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: grocery_non_food row 32</t>
+          <t>MISS OPR std SAT: Frozen</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: baby_kids row 33</t>
+          <t>MISS OPR std SAT: Non Food Retail</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: personal_care row 34</t>
+          <t>MISS OPR std SAT: News &amp; Mags</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OK waste: Produce = 888.48 row 37</t>
+          <t>OK OPR meat SAT: Beef = 12820.81 row 16</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: meat_total row 38</t>
+          <t>OK OPR meat SAT: Lamb = 1327.74 row 17</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>OK waste: dairy = 403.77 row 45</t>
+          <t>OK OPR meat SAT: Pork = 1766.48 row 18</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>OK waste: bread_cakes = 390.75 row 46</t>
+          <t>OK OPR meat SAT: Bacon &amp; Loose S.R.P = 1033.86 row 19</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>OK waste: Deli = 255.83 row 47</t>
+          <t>OK OPR meat SAT: Poultry = 13032.06 row 20</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OK waste: Provisions = 1000.74 row 48</t>
+          <t>OK OPR meat SAT: Fish = 5366.70 row 21</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OK waste: frozen = 96.81 row 49</t>
+          <t>SKIP waste top-section: grocery_impulse row 30</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OK waste: Beef = 64.49 row 39</t>
+          <t>SKIP waste top-section: grocery_edible row 31</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OK waste: Lamb = 38.36 row 40</t>
+          <t>OK waste: Produce = 707.32 row 37</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OK waste: Pork = 6.96 row 41</t>
+          <t>SKIP waste top-section: meat_total row 38</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OK waste: Bacon = 5.40 row 42</t>
+          <t>OK waste: dairy = 356.42 row 45</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OK waste: Poultry = 30.29 row 43</t>
+          <t>OK waste: bread_cakes = 362.86 row 46</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>OK waste: Fish = 522.70 row 44</t>
+          <t>OK waste: Deli = 241.38 row 47</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SKIP waste top-section: beer_wine_spirits row 35</t>
+          <t>OK waste: Provisions = 1195.74 row 48</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OK stocktake: Cigarettes = 131469.13 row 13</t>
+          <t>OK waste: frozen = 10.49 row 49</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OK stocktake: Produce = 11162.64 row 22</t>
+          <t>OK waste: Fish = 439.01 row 44</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OK stocktake: Fish = 1990.50 row 21</t>
+          <t>SKIP waste top-section: grocery_non_food row 32</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>OK stocktake: Beef = 11161.92 row 16</t>
+          <t>SKIP waste top-section: baby_kids row 33</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OK stocktake: Pork = 1209.33 row 18</t>
+          <t>SKIP waste top-section: personal_care row 34</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OK stocktake: Lamb = 1182.86 row 17</t>
+          <t>OK waste: Beef = 0.00 row 39</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OK stocktake: Poultry = 2228.00 row 20</t>
+          <t>OK waste: Lamb = 0.00 row 40</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>OK stocktake: Bacon &amp; Loose S.R.P = 512.42 row 19</t>
+          <t>OK waste: Pork = 0.00 row 41</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OK stocktake: Deli = 3880.07 row 23</t>
+          <t>OK waste: Bacon = 0.00 row 42</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OK stocktake: Provisions = 25129.61 row 24</t>
+          <t>OK waste: Poultry = 13.10 row 43</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OK sales inc vat G4: 394761.22</t>
+          <t>OK stocktake: Cigarettes = 141369.18 row 13</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>OK sales ex vat G5: 361766.91</t>
+          <t>OK stocktake: Produce = 11832.09 row 22</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OK margin G6: 0.1759</t>
+          <t>OK stocktake: Fish = 2177.42 row 21</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OK scan margin std row 13: 0.13</t>
+          <t>OK stocktake: Beef = 12611.55 row 16</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OK scan margin std row 22: 0.19</t>
+          <t>OK stocktake: Pork = 1244.26 row 18</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OK scan margin std row 23: 0.39</t>
+          <t>OK stocktake: Lamb = 1334.15 row 17</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>OK scan margin std row 24: 0.19</t>
+          <t>OK stocktake: Poultry = 3023.56 row 20</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 16: 0.19</t>
+          <t>OK stocktake: Bacon &amp; Loose S.R.P = 379.27 row 19</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 17: 0.24</t>
+          <t>OK stocktake: Deli = 3163.70 row 23</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 18: 0.21</t>
+          <t>OK stocktake: Provisions = 319.23 row 24</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 19: 0.11</t>
+          <t>OK sales inc vat G4: 374316.37</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>OK scan margin meat row 20: 0.17</t>
+          <t>OK sales ex vat G5: 344109.32</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
+        <is>
+          <t>OK margin G6: 0.1731</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 13: 0.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 22: 0.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 23: 0.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>OK scan margin std row 24: 0.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 16: 0.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 17: 0.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 18: 0.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 19: 0.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>OK scan margin meat row 20: 0.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>OK scan margin meat row 21: 0.18</t>
         </is>

</xml_diff>